<commit_message>
Afvulverslag: Global Keg-rijen vervangen door '20L Other kegs'
- Rij '20L Global Keg' verwijderd, '20L Global Keg (S)' hernoemd naar '20L Other kegs'
- Labels gelijkgetrokken: '20L KU Fust', '20L Gbr. Door Vrouwen fust'
- Alle verwijzingen onder de verwijderde rij meegeschoven (Afvulverslag-formules,
  Afvullen!C59/C60/E60/C61, conditional formatting, merges, dimension)
- fix-american-dates.js: Afvulverslag!D99 -> D98

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CvHodB7rajqHXKYMVFnfMs
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -29689,7 +29689,7 @@
       </c>
       <c r="B59" s="2067" t="n"/>
       <c r="C59" s="2074">
-        <f>Afvulverslag!M49</f>
+        <f>Afvulverslag!M48</f>
         <v/>
       </c>
       <c r="D59" s="2068" t="n"/>
@@ -29737,12 +29737,12 @@
       </c>
       <c r="B60" s="2069" t="n"/>
       <c r="C60" s="2076">
-        <f>Afvulverslag!M77</f>
+        <f>Afvulverslag!M76</f>
         <v/>
       </c>
       <c r="D60" s="2070" t="n"/>
       <c r="E60" s="2077">
-        <f>IFERROR(Afvulverslag!M82/Afvulverslag!K82,"")</f>
+        <f>IFERROR(Afvulverslag!M81/Afvulverslag!K81,"")</f>
         <v/>
       </c>
       <c r="F60" s="2070" t="n"/>
@@ -29784,7 +29784,7 @@
       </c>
       <c r="B61" s="2069" t="n"/>
       <c r="C61" s="2078">
-        <f>SUM(Afvulverslag!M86:M88)</f>
+        <f>SUM(Afvulverslag!M85:M87)</f>
         <v/>
       </c>
       <c r="D61" s="2070" t="n"/>
@@ -31093,7 +31093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R103"/>
+  <dimension ref="A1:R102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.00390625" defaultRowHeight="15" zeroHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="2.5" customWidth="1" style="2094" min="1" max="1"/>
@@ -31457,7 +31457,7 @@
       <c r="K11" s="1521" t="n"/>
       <c r="L11" s="1521" t="n"/>
       <c r="M11" s="2135">
-        <f>SUM(M34:M42)</f>
+        <f>SUM(M34:M41)</f>
         <v/>
       </c>
       <c r="N11" s="1075" t="n"/>
@@ -31513,7 +31513,7 @@
       <c r="K13" s="1521" t="n"/>
       <c r="L13" s="1521" t="n"/>
       <c r="M13" s="2139">
-        <f>SUM(K45:K47)</f>
+        <f>SUM(K44:K46)</f>
         <v/>
       </c>
       <c r="N13" s="2140" t="n"/>
@@ -32084,7 +32084,7 @@
     <row r="35" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B35" s="2013" t="inlineStr">
         <is>
-          <t>20L Jopen/KU Fust</t>
+          <t>20L KU Fust</t>
         </is>
       </c>
       <c r="C35" s="2149" t="n"/>
@@ -32170,7 +32170,7 @@
     <row r="39" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B39" s="2013" t="inlineStr">
         <is>
-          <t>20L Gbr, Door Vrouwen fust</t>
+          <t>20L Gbr. Door Vrouwen fust</t>
         </is>
       </c>
       <c r="C39" s="1521" t="n"/>
@@ -32194,7 +32194,7 @@
     <row r="40" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B40" s="2013" t="inlineStr">
         <is>
-          <t>20L Global Keg (S)</t>
+          <t>20L Other kegs</t>
         </is>
       </c>
       <c r="C40" s="1521" t="n"/>
@@ -32215,19 +32215,19 @@
         <v/>
       </c>
     </row>
-    <row r="41" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+    <row r="41" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B41" s="2013" t="inlineStr">
         <is>
-          <t>20L Global Keg</t>
+          <t>30L KeyKeg</t>
         </is>
       </c>
       <c r="C41" s="1521" t="n"/>
-      <c r="D41" s="2167" t="n"/>
-      <c r="E41" s="2151" t="n"/>
-      <c r="F41" s="2151" t="n"/>
-      <c r="G41" s="2151" t="n"/>
-      <c r="H41" s="2151" t="n"/>
-      <c r="I41" s="2150" t="n"/>
+      <c r="D41" s="2160" t="n"/>
+      <c r="E41" s="2160" t="n"/>
+      <c r="F41" s="2160" t="n"/>
+      <c r="G41" s="2160" t="n"/>
+      <c r="H41" s="2160" t="n"/>
+      <c r="I41" s="2161" t="n"/>
       <c r="J41" s="1521" t="n"/>
       <c r="K41" s="2152">
         <f>SUM(D41:I41)</f>
@@ -32235,102 +32235,102 @@
       </c>
       <c r="L41" s="2112" t="n"/>
       <c r="M41" s="2154">
-        <f>K41*20</f>
+        <f>K41*30</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B42" s="2013" t="inlineStr">
-        <is>
-          <t>30L KeyKeg</t>
-        </is>
-      </c>
-      <c r="C42" s="1521" t="n"/>
-      <c r="D42" s="2160" t="n"/>
-      <c r="E42" s="2160" t="n"/>
-      <c r="F42" s="2160" t="n"/>
-      <c r="G42" s="2160" t="n"/>
-      <c r="H42" s="2160" t="n"/>
-      <c r="I42" s="2161" t="n"/>
-      <c r="J42" s="1521" t="n"/>
-      <c r="K42" s="2152">
-        <f>SUM(D42:I42)</f>
-        <v/>
-      </c>
-      <c r="L42" s="2112" t="n"/>
-      <c r="M42" s="2154">
-        <f>K42*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B43" s="2168" t="n"/>
-      <c r="C43" s="1512" t="n"/>
-      <c r="D43" s="2169" t="n"/>
-      <c r="E43" s="2169" t="n"/>
-      <c r="F43" s="2169" t="n"/>
-      <c r="G43" s="2169" t="n"/>
-      <c r="H43" s="2169" t="n"/>
-      <c r="I43" s="2169" t="n"/>
-      <c r="J43" s="2170" t="n"/>
-      <c r="K43" s="2171" t="n"/>
-      <c r="L43" s="1521" t="n"/>
-      <c r="M43" s="1521" t="n"/>
-    </row>
-    <row r="44" outlineLevel="1" ht="55.5" customFormat="1" customHeight="1" s="1425">
-      <c r="B44" s="2172" t="inlineStr">
+      <c r="B42" s="2168" t="n"/>
+      <c r="C42" s="1512" t="n"/>
+      <c r="D42" s="2169" t="n"/>
+      <c r="E42" s="2169" t="n"/>
+      <c r="F42" s="2169" t="n"/>
+      <c r="G42" s="2169" t="n"/>
+      <c r="H42" s="2169" t="n"/>
+      <c r="I42" s="2169" t="n"/>
+      <c r="J42" s="2170" t="n"/>
+      <c r="K42" s="2171" t="n"/>
+      <c r="L42" s="1521" t="n"/>
+      <c r="M42" s="1521" t="n"/>
+    </row>
+    <row r="43" outlineLevel="1" ht="55.5" customFormat="1" customHeight="1" s="1425">
+      <c r="B43" s="2172" t="inlineStr">
         <is>
           <t>GEBRUIKT TBV SAMENVOEGEN / BARREL AGING</t>
         </is>
       </c>
-      <c r="C44" s="2147" t="inlineStr">
+      <c r="C43" s="2147" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
-      <c r="D44" s="2010" t="inlineStr">
+      <c r="D43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
-      <c r="E44" s="2010" t="inlineStr">
+      <c r="E43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
-      <c r="F44" s="2010" t="inlineStr">
+      <c r="F43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
-      <c r="G44" s="2010" t="inlineStr">
+      <c r="G43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
-      <c r="H44" s="2010" t="inlineStr">
+      <c r="H43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
-      <c r="I44" s="2010" t="inlineStr">
+      <c r="I43" s="2010" t="inlineStr">
         <is>
           <t>Liters</t>
         </is>
       </c>
+      <c r="J43" s="1521" t="n"/>
+      <c r="K43" s="2010" t="inlineStr">
+        <is>
+          <t>TOTALEN Liters</t>
+        </is>
+      </c>
+      <c r="L43" s="1114" t="n"/>
+      <c r="M43" s="1115" t="n"/>
+    </row>
+    <row r="44" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B44" s="2013" t="inlineStr">
+        <is>
+          <t>TBV BATCH …,</t>
+        </is>
+      </c>
+      <c r="C44" s="2150" t="n"/>
+      <c r="D44" s="2150" t="n"/>
+      <c r="E44" s="2150" t="n"/>
+      <c r="F44" s="2150" t="n"/>
+      <c r="G44" s="2150" t="n"/>
+      <c r="H44" s="2150" t="n"/>
+      <c r="I44" s="2150" t="n"/>
       <c r="J44" s="1521" t="n"/>
-      <c r="K44" s="2010" t="inlineStr">
-        <is>
-          <t>TOTALEN Liters</t>
-        </is>
-      </c>
-      <c r="L44" s="1114" t="n"/>
-      <c r="M44" s="1115" t="n"/>
+      <c r="K44" s="2152">
+        <f>SUM(D44:I44)</f>
+        <v/>
+      </c>
+      <c r="L44" s="2112" t="n"/>
+      <c r="M44" s="2154">
+        <f>K44</f>
+        <v/>
+      </c>
     </row>
     <row r="45" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B45" s="2013" t="inlineStr">
         <is>
-          <t>TBV BATCH …,</t>
+          <t>TBV BARREL AGING BATCH…</t>
         </is>
       </c>
       <c r="C45" s="2150" t="n"/>
@@ -32352,172 +32352,176 @@
       </c>
     </row>
     <row r="46" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B46" s="2013" t="inlineStr">
-        <is>
-          <t>TBV BARREL AGING BATCH…</t>
-        </is>
-      </c>
-      <c r="C46" s="2150" t="n"/>
-      <c r="D46" s="2150" t="n"/>
-      <c r="E46" s="2150" t="n"/>
-      <c r="F46" s="2150" t="n"/>
-      <c r="G46" s="2150" t="n"/>
-      <c r="H46" s="2150" t="n"/>
-      <c r="I46" s="2150" t="n"/>
+      <c r="B46" s="2013" t="n"/>
+      <c r="C46" s="2160" t="n"/>
+      <c r="D46" s="2160" t="n"/>
+      <c r="E46" s="2161" t="n"/>
+      <c r="F46" s="2161" t="n"/>
+      <c r="G46" s="2161" t="n"/>
+      <c r="H46" s="2161" t="n"/>
+      <c r="I46" s="2161" t="n"/>
       <c r="J46" s="1521" t="n"/>
       <c r="K46" s="2152">
         <f>SUM(D46:I46)</f>
         <v/>
       </c>
       <c r="L46" s="2112" t="n"/>
-      <c r="M46" s="2154">
-        <f>K46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B47" s="2013" t="n"/>
-      <c r="C47" s="2160" t="n"/>
-      <c r="D47" s="2160" t="n"/>
-      <c r="E47" s="2161" t="n"/>
-      <c r="F47" s="2161" t="n"/>
-      <c r="G47" s="2161" t="n"/>
-      <c r="H47" s="2161" t="n"/>
-      <c r="I47" s="2161" t="n"/>
-      <c r="J47" s="1521" t="n"/>
-      <c r="K47" s="2152">
-        <f>SUM(D47:I47)</f>
-        <v/>
-      </c>
-      <c r="L47" s="2112" t="n"/>
-      <c r="M47" s="2112" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="1339"/>
-    <row r="49" ht="23.25" customFormat="1" customHeight="1" s="1425">
-      <c r="B49" s="2173" t="inlineStr">
+      <c r="M46" s="2112" t="n"/>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="1339"/>
+    <row r="48" ht="23.25" customFormat="1" customHeight="1" s="1425">
+      <c r="B48" s="2173" t="inlineStr">
         <is>
           <t>VERBRUIKEN :</t>
         </is>
       </c>
-      <c r="C49" s="1114" t="n"/>
-      <c r="D49" s="1114" t="n"/>
-      <c r="E49" s="1114" t="n"/>
-      <c r="F49" s="1114" t="n"/>
-      <c r="G49" s="1114" t="n"/>
-      <c r="H49" s="1114" t="n"/>
-      <c r="I49" s="1115" t="n"/>
+      <c r="C48" s="1114" t="n"/>
+      <c r="D48" s="1114" t="n"/>
+      <c r="E48" s="1114" t="n"/>
+      <c r="F48" s="1114" t="n"/>
+      <c r="G48" s="1114" t="n"/>
+      <c r="H48" s="1114" t="n"/>
+      <c r="I48" s="1115" t="n"/>
+      <c r="J48" s="1521" t="n"/>
+      <c r="K48" s="2145" t="inlineStr">
+        <is>
+          <t>UITSCHRIJVEN (-)</t>
+        </is>
+      </c>
+      <c r="L48" s="1114" t="n"/>
+      <c r="M48" s="1115" t="n"/>
+      <c r="N48" s="1521" t="n"/>
+      <c r="O48" s="1521" t="n"/>
+      <c r="P48" s="1521" t="n"/>
+      <c r="Q48" s="1521" t="n"/>
+    </row>
+    <row r="49" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B49" s="2174" t="inlineStr">
+        <is>
+          <t>VERBRUIKEN FLES</t>
+        </is>
+      </c>
+      <c r="C49" s="2147" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+      <c r="D49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="E49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="F49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="G49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="H49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="I49" s="1137" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
       <c r="J49" s="1521" t="n"/>
-      <c r="K49" s="2145" t="inlineStr">
-        <is>
-          <t>UITSCHRIJVEN (-)</t>
-        </is>
-      </c>
-      <c r="L49" s="1114" t="n"/>
-      <c r="M49" s="1115" t="n"/>
+      <c r="K49" s="2175" t="inlineStr">
+        <is>
+          <t>TOTALEN</t>
+        </is>
+      </c>
+      <c r="L49" s="2036" t="n"/>
+      <c r="M49" s="2148" t="inlineStr">
+        <is>
+          <t>VERLIES</t>
+        </is>
+      </c>
       <c r="N49" s="1521" t="n"/>
       <c r="O49" s="1521" t="n"/>
       <c r="P49" s="1521" t="n"/>
       <c r="Q49" s="1521" t="n"/>
     </row>
-    <row r="50" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B50" s="2174" t="inlineStr">
-        <is>
-          <t>VERBRUIKEN FLES</t>
-        </is>
-      </c>
-      <c r="C50" s="2147" t="inlineStr">
-        <is>
-          <t>Opmerkingen</t>
-        </is>
-      </c>
-      <c r="D50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="E50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="F50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="G50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="H50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="I50" s="1137" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
+    <row r="50" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B50" s="2016" t="inlineStr">
+        <is>
+          <t>Fles 33cl</t>
+        </is>
+      </c>
+      <c r="C50" s="2176" t="n"/>
+      <c r="D50" s="2165" t="n"/>
+      <c r="E50" s="2166" t="n"/>
+      <c r="F50" s="2166" t="n"/>
+      <c r="G50" s="2166" t="n"/>
+      <c r="H50" s="2166" t="n"/>
+      <c r="I50" s="2166" t="n"/>
       <c r="J50" s="1521" t="n"/>
-      <c r="K50" s="2175" t="inlineStr">
-        <is>
-          <t>TOTALEN</t>
-        </is>
-      </c>
-      <c r="L50" s="2036" t="n"/>
-      <c r="M50" s="2148" t="inlineStr">
-        <is>
-          <t>VERLIES</t>
-        </is>
+      <c r="K50" s="2152">
+        <f>SUM(D50:I50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="2112" t="n"/>
+      <c r="M50" s="2177">
+        <f>K50-SUM(K17:K18)*24-SUM(K20:K21)*12</f>
+        <v/>
       </c>
       <c r="N50" s="1521" t="n"/>
       <c r="O50" s="1521" t="n"/>
       <c r="P50" s="1521" t="n"/>
       <c r="Q50" s="1521" t="n"/>
     </row>
-    <row r="51" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B51" s="2016" t="inlineStr">
-        <is>
-          <t>Fles 33cl</t>
-        </is>
-      </c>
-      <c r="C51" s="2176" t="n"/>
-      <c r="D51" s="2165" t="n"/>
-      <c r="E51" s="2166" t="n"/>
-      <c r="F51" s="2166" t="n"/>
-      <c r="G51" s="2166" t="n"/>
-      <c r="H51" s="2166" t="n"/>
-      <c r="I51" s="2166" t="n"/>
+    <row r="51" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B51" s="2178" t="n"/>
+      <c r="C51" s="2163" t="n"/>
+      <c r="D51" s="2163" t="n"/>
+      <c r="E51" s="2163" t="n"/>
+      <c r="F51" s="2163" t="n"/>
+      <c r="G51" s="2163" t="n"/>
+      <c r="H51" s="2163" t="n"/>
+      <c r="I51" s="2163" t="n"/>
       <c r="J51" s="1521" t="n"/>
-      <c r="K51" s="2152">
-        <f>SUM(D51:I51)</f>
-        <v/>
-      </c>
+      <c r="K51" s="2152" t="n"/>
       <c r="L51" s="2112" t="n"/>
-      <c r="M51" s="2177">
-        <f>K51-SUM(K17:K18)*24-SUM(K20:K21)*12</f>
-        <v/>
-      </c>
+      <c r="M51" s="2177" t="n"/>
       <c r="N51" s="1521" t="n"/>
       <c r="O51" s="1521" t="n"/>
       <c r="P51" s="1521" t="n"/>
       <c r="Q51" s="1521" t="n"/>
     </row>
-    <row r="52" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B52" s="2178" t="n"/>
-      <c r="C52" s="2163" t="n"/>
-      <c r="D52" s="2163" t="n"/>
-      <c r="E52" s="2163" t="n"/>
-      <c r="F52" s="2163" t="n"/>
-      <c r="G52" s="2163" t="n"/>
-      <c r="H52" s="2163" t="n"/>
-      <c r="I52" s="2163" t="n"/>
+    <row r="52" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B52" s="2016" t="inlineStr">
+        <is>
+          <t>Stickerlabel 33cl - Main</t>
+        </is>
+      </c>
+      <c r="C52" s="2179" t="n"/>
+      <c r="D52" s="2165" t="n"/>
+      <c r="E52" s="2166" t="n"/>
+      <c r="F52" s="2166" t="n"/>
+      <c r="G52" s="2166" t="n"/>
+      <c r="H52" s="2166" t="n"/>
+      <c r="I52" s="2166" t="n"/>
       <c r="J52" s="1521" t="n"/>
-      <c r="K52" s="2152" t="n"/>
+      <c r="K52" s="2152">
+        <f>SUM(D52:I52)</f>
+        <v/>
+      </c>
       <c r="L52" s="2112" t="n"/>
-      <c r="M52" s="2177" t="n"/>
+      <c r="M52" s="2177">
+        <f>K52-$K$17*24-$K$20*12</f>
+        <v/>
+      </c>
       <c r="N52" s="1521" t="n"/>
       <c r="O52" s="1521" t="n"/>
       <c r="P52" s="1521" t="n"/>
@@ -32526,16 +32530,16 @@
     <row r="53" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B53" s="2016" t="inlineStr">
         <is>
-          <t>Stickerlabel 33cl - Main</t>
-        </is>
-      </c>
-      <c r="C53" s="2179" t="n"/>
-      <c r="D53" s="2165" t="n"/>
-      <c r="E53" s="2166" t="n"/>
-      <c r="F53" s="2166" t="n"/>
-      <c r="G53" s="2166" t="n"/>
-      <c r="H53" s="2166" t="n"/>
-      <c r="I53" s="2166" t="n"/>
+          <t>Stickerlabel 33cl - Neck</t>
+        </is>
+      </c>
+      <c r="C53" s="2161" t="n"/>
+      <c r="D53" s="2160" t="n"/>
+      <c r="E53" s="2161" t="n"/>
+      <c r="F53" s="2161" t="n"/>
+      <c r="G53" s="2161" t="n"/>
+      <c r="H53" s="2161" t="n"/>
+      <c r="I53" s="2161" t="n"/>
       <c r="J53" s="1521" t="n"/>
       <c r="K53" s="2152">
         <f>SUM(D53:I53)</f>
@@ -32551,47 +32555,47 @@
       <c r="P53" s="1521" t="n"/>
       <c r="Q53" s="1521" t="n"/>
     </row>
-    <row r="54" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B54" s="2016" t="inlineStr">
-        <is>
-          <t>Stickerlabel 33cl - Neck</t>
-        </is>
-      </c>
-      <c r="C54" s="2161" t="n"/>
-      <c r="D54" s="2160" t="n"/>
-      <c r="E54" s="2161" t="n"/>
-      <c r="F54" s="2161" t="n"/>
-      <c r="G54" s="2161" t="n"/>
-      <c r="H54" s="2161" t="n"/>
-      <c r="I54" s="2161" t="n"/>
+    <row r="54" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B54" s="1099" t="n"/>
+      <c r="C54" s="2170" t="n"/>
+      <c r="D54" s="1521" t="n"/>
+      <c r="E54" s="1521" t="n"/>
+      <c r="F54" s="1521" t="n"/>
+      <c r="G54" s="1521" t="n"/>
+      <c r="H54" s="1521" t="n"/>
+      <c r="I54" s="1521" t="n"/>
       <c r="J54" s="1521" t="n"/>
-      <c r="K54" s="2152">
-        <f>SUM(D54:I54)</f>
-        <v/>
-      </c>
+      <c r="K54" s="2152" t="n"/>
       <c r="L54" s="2112" t="n"/>
-      <c r="M54" s="2177">
-        <f>K54-$K$17*24-$K$20*12</f>
-        <v/>
-      </c>
+      <c r="M54" s="2177" t="n"/>
       <c r="N54" s="1521" t="n"/>
       <c r="O54" s="1521" t="n"/>
       <c r="P54" s="1521" t="n"/>
       <c r="Q54" s="1521" t="n"/>
     </row>
-    <row r="55" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B55" s="1099" t="n"/>
-      <c r="C55" s="2170" t="n"/>
-      <c r="D55" s="1521" t="n"/>
-      <c r="E55" s="1521" t="n"/>
-      <c r="F55" s="1521" t="n"/>
-      <c r="G55" s="1521" t="n"/>
-      <c r="H55" s="1521" t="n"/>
-      <c r="I55" s="1521" t="n"/>
+    <row r="55" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B55" s="2016" t="inlineStr">
+        <is>
+          <t>Omdozen 24x33cl - Bedrukt:</t>
+        </is>
+      </c>
+      <c r="C55" s="2179" t="n"/>
+      <c r="D55" s="2165" t="n"/>
+      <c r="E55" s="2166" t="n"/>
+      <c r="F55" s="2166" t="n"/>
+      <c r="G55" s="2166" t="n"/>
+      <c r="H55" s="2166" t="n"/>
+      <c r="I55" s="2166" t="n"/>
       <c r="J55" s="1521" t="n"/>
-      <c r="K55" s="2152" t="n"/>
+      <c r="K55" s="2152">
+        <f>SUM(D55:I55)</f>
+        <v/>
+      </c>
       <c r="L55" s="2112" t="n"/>
-      <c r="M55" s="2177" t="n"/>
+      <c r="M55" s="2152">
+        <f>K55-K17</f>
+        <v/>
+      </c>
       <c r="N55" s="1521" t="n"/>
       <c r="O55" s="1521" t="n"/>
       <c r="P55" s="1521" t="n"/>
@@ -32600,16 +32604,16 @@
     <row r="56" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B56" s="2016" t="inlineStr">
         <is>
-          <t>Omdozen 24x33cl - Bedrukt:</t>
-        </is>
-      </c>
-      <c r="C56" s="2179" t="n"/>
-      <c r="D56" s="2165" t="n"/>
-      <c r="E56" s="2166" t="n"/>
-      <c r="F56" s="2166" t="n"/>
-      <c r="G56" s="2166" t="n"/>
-      <c r="H56" s="2166" t="n"/>
-      <c r="I56" s="2166" t="n"/>
+          <t>Omdozen 24x33cl - Blanco</t>
+        </is>
+      </c>
+      <c r="C56" s="2180" t="n"/>
+      <c r="D56" s="2160" t="n"/>
+      <c r="E56" s="2161" t="n"/>
+      <c r="F56" s="2161" t="n"/>
+      <c r="G56" s="2161" t="n"/>
+      <c r="H56" s="2161" t="n"/>
+      <c r="I56" s="2161" t="n"/>
       <c r="J56" s="1521" t="n"/>
       <c r="K56" s="2152">
         <f>SUM(D56:I56)</f>
@@ -32617,7 +32621,7 @@
       </c>
       <c r="L56" s="2112" t="n"/>
       <c r="M56" s="2152">
-        <f>K56-K17</f>
+        <f>K56-K18</f>
         <v/>
       </c>
       <c r="N56" s="1521" t="n"/>
@@ -32626,46 +32630,46 @@
       <c r="Q56" s="1521" t="n"/>
     </row>
     <row r="57" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B57" s="2016" t="inlineStr">
-        <is>
-          <t>Omdozen 24x33cl - Blanco</t>
-        </is>
-      </c>
-      <c r="C57" s="2180" t="n"/>
-      <c r="D57" s="2160" t="n"/>
-      <c r="E57" s="2161" t="n"/>
-      <c r="F57" s="2161" t="n"/>
-      <c r="G57" s="2161" t="n"/>
-      <c r="H57" s="2161" t="n"/>
-      <c r="I57" s="2161" t="n"/>
+      <c r="B57" s="1099" t="n"/>
+      <c r="C57" s="1521" t="n"/>
+      <c r="D57" s="1521" t="n"/>
+      <c r="E57" s="1521" t="n"/>
+      <c r="F57" s="1521" t="n"/>
+      <c r="G57" s="1521" t="n"/>
+      <c r="H57" s="1521" t="n"/>
+      <c r="I57" s="1521" t="n"/>
       <c r="J57" s="1521" t="n"/>
-      <c r="K57" s="2152">
-        <f>SUM(D57:I57)</f>
-        <v/>
-      </c>
+      <c r="K57" s="2152" t="n"/>
       <c r="L57" s="2112" t="n"/>
-      <c r="M57" s="2152">
-        <f>K57-K18</f>
-        <v/>
-      </c>
+      <c r="M57" s="2177" t="n"/>
       <c r="N57" s="1521" t="n"/>
       <c r="O57" s="1521" t="n"/>
       <c r="P57" s="1521" t="n"/>
       <c r="Q57" s="1521" t="n"/>
     </row>
     <row r="58" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B58" s="1099" t="n"/>
-      <c r="C58" s="1521" t="n"/>
-      <c r="D58" s="1521" t="n"/>
-      <c r="E58" s="1521" t="n"/>
-      <c r="F58" s="1521" t="n"/>
-      <c r="G58" s="1521" t="n"/>
-      <c r="H58" s="1521" t="n"/>
-      <c r="I58" s="1521" t="n"/>
+      <c r="B58" s="2016" t="inlineStr">
+        <is>
+          <t>Omdozen 12x33cl - Bedrukt:</t>
+        </is>
+      </c>
+      <c r="C58" s="2179" t="n"/>
+      <c r="D58" s="2165" t="n"/>
+      <c r="E58" s="2166" t="n"/>
+      <c r="F58" s="2166" t="n"/>
+      <c r="G58" s="2166" t="n"/>
+      <c r="H58" s="2166" t="n"/>
+      <c r="I58" s="2166" t="n"/>
       <c r="J58" s="1521" t="n"/>
-      <c r="K58" s="2152" t="n"/>
+      <c r="K58" s="2152">
+        <f>SUM(D58:I58)</f>
+        <v/>
+      </c>
       <c r="L58" s="2112" t="n"/>
-      <c r="M58" s="2177" t="n"/>
+      <c r="M58" s="2152">
+        <f>K58-K20</f>
+        <v/>
+      </c>
       <c r="N58" s="1521" t="n"/>
       <c r="O58" s="1521" t="n"/>
       <c r="P58" s="1521" t="n"/>
@@ -32674,16 +32678,16 @@
     <row r="59" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B59" s="2016" t="inlineStr">
         <is>
-          <t>Omdozen 12x33cl - Bedrukt:</t>
-        </is>
-      </c>
-      <c r="C59" s="2179" t="n"/>
-      <c r="D59" s="2165" t="n"/>
-      <c r="E59" s="2166" t="n"/>
-      <c r="F59" s="2166" t="n"/>
-      <c r="G59" s="2166" t="n"/>
-      <c r="H59" s="2166" t="n"/>
-      <c r="I59" s="2166" t="n"/>
+          <t>Omdozen 12x33cl - Blanco</t>
+        </is>
+      </c>
+      <c r="C59" s="2180" t="n"/>
+      <c r="D59" s="2160" t="n"/>
+      <c r="E59" s="2161" t="n"/>
+      <c r="F59" s="2161" t="n"/>
+      <c r="G59" s="2161" t="n"/>
+      <c r="H59" s="2161" t="n"/>
+      <c r="I59" s="2161" t="n"/>
       <c r="J59" s="1521" t="n"/>
       <c r="K59" s="2152">
         <f>SUM(D59:I59)</f>
@@ -32691,7 +32695,7 @@
       </c>
       <c r="L59" s="2112" t="n"/>
       <c r="M59" s="2152">
-        <f>K59-K20</f>
+        <f>K59-K21</f>
         <v/>
       </c>
       <c r="N59" s="1521" t="n"/>
@@ -32700,122 +32704,122 @@
       <c r="Q59" s="1521" t="n"/>
     </row>
     <row r="60" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B60" s="2016" t="inlineStr">
-        <is>
-          <t>Omdozen 12x33cl - Blanco</t>
-        </is>
-      </c>
-      <c r="C60" s="2180" t="n"/>
-      <c r="D60" s="2160" t="n"/>
-      <c r="E60" s="2161" t="n"/>
-      <c r="F60" s="2161" t="n"/>
-      <c r="G60" s="2161" t="n"/>
-      <c r="H60" s="2161" t="n"/>
-      <c r="I60" s="2161" t="n"/>
+      <c r="B60" s="1099" t="n"/>
+      <c r="C60" s="2170" t="n"/>
+      <c r="D60" s="1521" t="n"/>
+      <c r="E60" s="1521" t="n"/>
+      <c r="F60" s="1521" t="n"/>
+      <c r="G60" s="1521" t="n"/>
+      <c r="H60" s="1521" t="n"/>
+      <c r="I60" s="1521" t="n"/>
       <c r="J60" s="1521" t="n"/>
-      <c r="K60" s="2152">
-        <f>SUM(D60:I60)</f>
-        <v/>
-      </c>
+      <c r="K60" s="2152" t="n"/>
       <c r="L60" s="2112" t="n"/>
-      <c r="M60" s="2152">
-        <f>K60-K21</f>
-        <v/>
-      </c>
+      <c r="M60" s="2177" t="n"/>
       <c r="N60" s="1521" t="n"/>
       <c r="O60" s="1521" t="n"/>
       <c r="P60" s="1521" t="n"/>
       <c r="Q60" s="1521" t="n"/>
     </row>
     <row r="61" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B61" s="1099" t="n"/>
-      <c r="C61" s="2170" t="n"/>
-      <c r="D61" s="1521" t="n"/>
-      <c r="E61" s="1521" t="n"/>
-      <c r="F61" s="1521" t="n"/>
-      <c r="G61" s="1521" t="n"/>
-      <c r="H61" s="1521" t="n"/>
-      <c r="I61" s="1521" t="n"/>
+      <c r="B61" s="2016" t="inlineStr">
+        <is>
+          <t>Kroonkurk:</t>
+        </is>
+      </c>
+      <c r="C61" s="2181" t="n"/>
+      <c r="D61" s="2137" t="n"/>
+      <c r="E61" s="2138" t="n"/>
+      <c r="F61" s="2138" t="n"/>
+      <c r="G61" s="2138" t="n"/>
+      <c r="H61" s="2138" t="n"/>
+      <c r="I61" s="2138" t="n"/>
       <c r="J61" s="1521" t="n"/>
-      <c r="K61" s="2152" t="n"/>
+      <c r="K61" s="2152">
+        <f>SUM(D61:I61)</f>
+        <v/>
+      </c>
       <c r="L61" s="2112" t="n"/>
-      <c r="M61" s="2177" t="n"/>
+      <c r="M61" s="2152">
+        <f>C61-SUM(K17:K18)*24-SUM(K20:K21)*12</f>
+        <v/>
+      </c>
       <c r="N61" s="1521" t="n"/>
-      <c r="O61" s="1521" t="n"/>
+      <c r="O61" s="1521" t="inlineStr">
+        <is>
+          <t>Doos á</t>
+        </is>
+      </c>
       <c r="P61" s="1521" t="n"/>
-      <c r="Q61" s="1521" t="n"/>
-    </row>
-    <row r="62" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B62" s="2016" t="inlineStr">
-        <is>
-          <t>Kroonkurk:</t>
-        </is>
-      </c>
-      <c r="C62" s="2181" t="n"/>
-      <c r="D62" s="2137" t="n"/>
-      <c r="E62" s="2138" t="n"/>
-      <c r="F62" s="2138" t="n"/>
-      <c r="G62" s="2138" t="n"/>
-      <c r="H62" s="2138" t="n"/>
-      <c r="I62" s="2138" t="n"/>
+      <c r="Q61" s="2137" t="n">
+        <v>10000</v>
+      </c>
+      <c r="R61" s="2125">
+        <f>K61/Q61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B62" s="1099" t="n"/>
+      <c r="C62" s="1521" t="n"/>
+      <c r="D62" s="1521" t="n"/>
+      <c r="E62" s="1521" t="n"/>
+      <c r="F62" s="1521" t="n"/>
+      <c r="G62" s="1521" t="n"/>
+      <c r="H62" s="1521" t="n"/>
+      <c r="I62" s="1521" t="n"/>
       <c r="J62" s="1521" t="n"/>
-      <c r="K62" s="2152">
-        <f>SUM(D62:I62)</f>
-        <v/>
-      </c>
+      <c r="K62" s="2152" t="n"/>
       <c r="L62" s="2112" t="n"/>
-      <c r="M62" s="2152">
-        <f>C62-SUM(K17:K18)*24-SUM(K20:K21)*12</f>
-        <v/>
-      </c>
+      <c r="M62" s="2177" t="n"/>
       <c r="N62" s="1521" t="n"/>
-      <c r="O62" s="1521" t="inlineStr">
-        <is>
-          <t>Doos á</t>
-        </is>
-      </c>
-      <c r="P62" s="1521" t="n"/>
-      <c r="Q62" s="2137" t="n">
-        <v>10000</v>
-      </c>
-      <c r="R62" s="2125">
-        <f>K62/Q62</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B63" s="1099" t="n"/>
-      <c r="C63" s="1521" t="n"/>
-      <c r="D63" s="1521" t="n"/>
-      <c r="E63" s="1521" t="n"/>
-      <c r="F63" s="1521" t="n"/>
-      <c r="G63" s="1521" t="n"/>
-      <c r="H63" s="1521" t="n"/>
-      <c r="I63" s="1521" t="n"/>
+      <c r="O62" s="2182" t="inlineStr">
+        <is>
+          <t>Inhoud doos kan variëren!</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B63" s="2016" t="inlineStr">
+        <is>
+          <t>Fles 75cl</t>
+        </is>
+      </c>
+      <c r="C63" s="2179" t="n"/>
+      <c r="D63" s="2165" t="n"/>
+      <c r="E63" s="2166" t="n"/>
+      <c r="F63" s="2166" t="n"/>
+      <c r="G63" s="2166" t="n"/>
+      <c r="H63" s="2166" t="n"/>
+      <c r="I63" s="2166" t="n"/>
       <c r="J63" s="1521" t="n"/>
-      <c r="K63" s="2152" t="n"/>
+      <c r="K63" s="2152">
+        <f>SUM(D63:I63)</f>
+        <v/>
+      </c>
       <c r="L63" s="2112" t="n"/>
-      <c r="M63" s="2177" t="n"/>
+      <c r="M63" s="2177">
+        <f>K63-SUM(K23:K24)*6-K25*12</f>
+        <v/>
+      </c>
       <c r="N63" s="1521" t="n"/>
-      <c r="O63" s="2182" t="inlineStr">
-        <is>
-          <t>Inhoud doos kan variëren!</t>
-        </is>
-      </c>
+      <c r="O63" s="1521" t="n"/>
+      <c r="P63" s="1521" t="n"/>
+      <c r="Q63" s="1521" t="n"/>
     </row>
     <row r="64" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B64" s="2016" t="inlineStr">
         <is>
-          <t>Fles 75cl</t>
-        </is>
-      </c>
-      <c r="C64" s="2179" t="n"/>
-      <c r="D64" s="2165" t="n"/>
-      <c r="E64" s="2166" t="n"/>
-      <c r="F64" s="2166" t="n"/>
-      <c r="G64" s="2166" t="n"/>
-      <c r="H64" s="2166" t="n"/>
-      <c r="I64" s="2166" t="n"/>
+          <t>Stickerlabel 75cl - Main</t>
+        </is>
+      </c>
+      <c r="C64" s="2183" t="n"/>
+      <c r="D64" s="2151" t="n"/>
+      <c r="E64" s="2150" t="n"/>
+      <c r="F64" s="2150" t="n"/>
+      <c r="G64" s="2150" t="n"/>
+      <c r="H64" s="2150" t="n"/>
+      <c r="I64" s="2150" t="n"/>
       <c r="J64" s="1521" t="n"/>
       <c r="K64" s="2152">
         <f>SUM(D64:I64)</f>
@@ -32823,7 +32827,7 @@
       </c>
       <c r="L64" s="2112" t="n"/>
       <c r="M64" s="2177">
-        <f>K64-SUM(K23:K24)*6-K25*12</f>
+        <f>K64-K23*6</f>
         <v/>
       </c>
       <c r="N64" s="1521" t="n"/>
@@ -32834,16 +32838,16 @@
     <row r="65" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B65" s="2016" t="inlineStr">
         <is>
-          <t>Stickerlabel 75cl - Main</t>
+          <t>Stickerlabel 75cl - Neck</t>
         </is>
       </c>
       <c r="C65" s="2183" t="n"/>
-      <c r="D65" s="2151" t="n"/>
-      <c r="E65" s="2150" t="n"/>
-      <c r="F65" s="2150" t="n"/>
-      <c r="G65" s="2150" t="n"/>
-      <c r="H65" s="2150" t="n"/>
-      <c r="I65" s="2150" t="n"/>
+      <c r="D65" s="2167" t="n"/>
+      <c r="E65" s="2184" t="n"/>
+      <c r="F65" s="2184" t="n"/>
+      <c r="G65" s="2184" t="n"/>
+      <c r="H65" s="2184" t="n"/>
+      <c r="I65" s="2184" t="n"/>
       <c r="J65" s="1521" t="n"/>
       <c r="K65" s="2152">
         <f>SUM(D65:I65)</f>
@@ -32860,46 +32864,46 @@
       <c r="Q65" s="1521" t="n"/>
     </row>
     <row r="66" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B66" s="2016" t="inlineStr">
-        <is>
-          <t>Stickerlabel 75cl - Neck</t>
-        </is>
-      </c>
-      <c r="C66" s="2183" t="n"/>
-      <c r="D66" s="2167" t="n"/>
-      <c r="E66" s="2184" t="n"/>
-      <c r="F66" s="2184" t="n"/>
-      <c r="G66" s="2184" t="n"/>
-      <c r="H66" s="2184" t="n"/>
-      <c r="I66" s="2184" t="n"/>
+      <c r="B66" s="2185" t="n"/>
+      <c r="C66" s="2186" t="n"/>
+      <c r="D66" s="2187" t="n"/>
+      <c r="E66" s="2187" t="n"/>
+      <c r="F66" s="2187" t="n"/>
+      <c r="G66" s="2187" t="n"/>
+      <c r="H66" s="2187" t="n"/>
+      <c r="I66" s="2187" t="n"/>
       <c r="J66" s="1521" t="n"/>
-      <c r="K66" s="2152">
-        <f>SUM(D66:I66)</f>
-        <v/>
-      </c>
+      <c r="K66" s="2152" t="n"/>
       <c r="L66" s="2112" t="n"/>
-      <c r="M66" s="2177">
-        <f>K66-K23*6</f>
-        <v/>
-      </c>
+      <c r="M66" s="2177" t="n"/>
       <c r="N66" s="1521" t="n"/>
       <c r="O66" s="1521" t="n"/>
       <c r="P66" s="1521" t="n"/>
       <c r="Q66" s="1521" t="n"/>
     </row>
     <row r="67" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B67" s="2185" t="n"/>
-      <c r="C67" s="2186" t="n"/>
-      <c r="D67" s="2187" t="n"/>
-      <c r="E67" s="2187" t="n"/>
-      <c r="F67" s="2187" t="n"/>
-      <c r="G67" s="2187" t="n"/>
-      <c r="H67" s="2187" t="n"/>
-      <c r="I67" s="2187" t="n"/>
+      <c r="B67" s="2016" t="inlineStr">
+        <is>
+          <t>Omdozen 6x75cl - Bedrukt:</t>
+        </is>
+      </c>
+      <c r="C67" s="2179" t="n"/>
+      <c r="D67" s="2165" t="n"/>
+      <c r="E67" s="2166" t="n"/>
+      <c r="F67" s="2166" t="n"/>
+      <c r="G67" s="2166" t="n"/>
+      <c r="H67" s="2166" t="n"/>
+      <c r="I67" s="2166" t="n"/>
       <c r="J67" s="1521" t="n"/>
-      <c r="K67" s="2152" t="n"/>
+      <c r="K67" s="2152">
+        <f>SUM(D67:I67)</f>
+        <v/>
+      </c>
       <c r="L67" s="2112" t="n"/>
-      <c r="M67" s="2177" t="n"/>
+      <c r="M67" s="2152">
+        <f>K67-K23</f>
+        <v/>
+      </c>
       <c r="N67" s="1521" t="n"/>
       <c r="O67" s="1521" t="n"/>
       <c r="P67" s="1521" t="n"/>
@@ -32908,16 +32912,16 @@
     <row r="68" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B68" s="2016" t="inlineStr">
         <is>
-          <t>Omdozen 6x75cl - Bedrukt:</t>
-        </is>
-      </c>
-      <c r="C68" s="2179" t="n"/>
-      <c r="D68" s="2165" t="n"/>
-      <c r="E68" s="2166" t="n"/>
-      <c r="F68" s="2166" t="n"/>
-      <c r="G68" s="2166" t="n"/>
-      <c r="H68" s="2166" t="n"/>
-      <c r="I68" s="2166" t="n"/>
+          <t>Omdozen 6x75cl - Blanco</t>
+        </is>
+      </c>
+      <c r="C68" s="2188" t="n"/>
+      <c r="D68" s="2160" t="n"/>
+      <c r="E68" s="2161" t="n"/>
+      <c r="F68" s="2161" t="n"/>
+      <c r="G68" s="2161" t="n"/>
+      <c r="H68" s="2161" t="n"/>
+      <c r="I68" s="2161" t="n"/>
       <c r="J68" s="1521" t="n"/>
       <c r="K68" s="2152">
         <f>SUM(D68:I68)</f>
@@ -32925,7 +32929,7 @@
       </c>
       <c r="L68" s="2112" t="n"/>
       <c r="M68" s="2152">
-        <f>K68-K23</f>
+        <f>K68-K24</f>
         <v/>
       </c>
       <c r="N68" s="1521" t="n"/>
@@ -32934,72 +32938,82 @@
       <c r="Q68" s="1521" t="n"/>
     </row>
     <row r="69" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B69" s="2016" t="inlineStr">
-        <is>
-          <t>Omdozen 6x75cl - Blanco</t>
-        </is>
-      </c>
-      <c r="C69" s="2188" t="n"/>
-      <c r="D69" s="2160" t="n"/>
-      <c r="E69" s="2161" t="n"/>
-      <c r="F69" s="2161" t="n"/>
-      <c r="G69" s="2161" t="n"/>
-      <c r="H69" s="2161" t="n"/>
-      <c r="I69" s="2161" t="n"/>
+      <c r="B69" s="1099" t="n"/>
+      <c r="C69" s="2170" t="n"/>
+      <c r="D69" s="1521" t="n"/>
+      <c r="E69" s="1521" t="n"/>
+      <c r="F69" s="1521" t="n"/>
+      <c r="G69" s="1521" t="n"/>
+      <c r="H69" s="1521" t="n"/>
+      <c r="I69" s="1521" t="n"/>
       <c r="J69" s="1521" t="n"/>
-      <c r="K69" s="2152">
-        <f>SUM(D69:I69)</f>
-        <v/>
-      </c>
+      <c r="K69" s="2152" t="n"/>
       <c r="L69" s="2112" t="n"/>
-      <c r="M69" s="2152">
-        <f>K69-K24</f>
-        <v/>
-      </c>
+      <c r="M69" s="2152" t="n"/>
       <c r="N69" s="1521" t="n"/>
       <c r="O69" s="1521" t="n"/>
       <c r="P69" s="1521" t="n"/>
       <c r="Q69" s="1521" t="n"/>
     </row>
     <row r="70" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B70" s="1099" t="n"/>
-      <c r="C70" s="2170" t="n"/>
-      <c r="D70" s="1521" t="n"/>
-      <c r="E70" s="1521" t="n"/>
-      <c r="F70" s="1521" t="n"/>
-      <c r="G70" s="1521" t="n"/>
-      <c r="H70" s="1521" t="n"/>
-      <c r="I70" s="1521" t="n"/>
+      <c r="B70" s="2016" t="inlineStr">
+        <is>
+          <t>Kurk:</t>
+        </is>
+      </c>
+      <c r="C70" s="2179" t="n"/>
+      <c r="D70" s="2165" t="n"/>
+      <c r="E70" s="2166" t="n"/>
+      <c r="F70" s="2166" t="n"/>
+      <c r="G70" s="2166" t="n"/>
+      <c r="H70" s="2166" t="n"/>
+      <c r="I70" s="2166" t="n"/>
       <c r="J70" s="1521" t="n"/>
-      <c r="K70" s="2152" t="n"/>
+      <c r="K70" s="2152">
+        <f>SUM(D70:I70)</f>
+        <v/>
+      </c>
       <c r="L70" s="2112" t="n"/>
-      <c r="M70" s="2152" t="n"/>
+      <c r="M70" s="2152">
+        <f>K70-SUM(K23:K24)*6-K25*12</f>
+        <v/>
+      </c>
       <c r="N70" s="1521" t="n"/>
-      <c r="O70" s="1521" t="n"/>
+      <c r="O70" s="1521" t="inlineStr">
+        <is>
+          <t>Doos á</t>
+        </is>
+      </c>
       <c r="P70" s="1521" t="n"/>
-      <c r="Q70" s="1521" t="n"/>
+      <c r="Q70" s="2189" t="n">
+        <v>2500</v>
+      </c>
+      <c r="R70" s="2125">
+        <f>K70/Q70</f>
+        <v/>
+      </c>
     </row>
     <row r="71" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B71" s="2016" t="inlineStr">
         <is>
-          <t>Kurk:</t>
-        </is>
-      </c>
-      <c r="C71" s="2179" t="n"/>
-      <c r="D71" s="2165" t="n"/>
-      <c r="E71" s="2166" t="n"/>
-      <c r="F71" s="2166" t="n"/>
-      <c r="G71" s="2166" t="n"/>
-      <c r="H71" s="2166" t="n"/>
-      <c r="I71" s="2166" t="n"/>
-      <c r="J71" s="1521" t="n"/>
+          <t>Musseletten:</t>
+        </is>
+      </c>
+      <c r="C71" s="2188" t="n"/>
+      <c r="D71" s="2160" t="n"/>
+      <c r="E71" s="2161" t="n"/>
+      <c r="F71" s="2161" t="n"/>
+      <c r="G71" s="2161" t="n"/>
+      <c r="H71" s="2161" t="n"/>
+      <c r="I71" s="2161" t="n"/>
+      <c r="J71" s="2170" t="n"/>
       <c r="K71" s="2152">
         <f>SUM(D71:I71)</f>
         <v/>
       </c>
       <c r="L71" s="2112" t="n"/>
       <c r="M71" s="2152">
-        <f>K71-SUM(K23:K24)*6-K25*12</f>
+        <f>K71-SUM(K23:K24)*6--K25*12</f>
         <v/>
       </c>
       <c r="N71" s="1521" t="n"/>
@@ -33010,122 +33024,113 @@
       </c>
       <c r="P71" s="1521" t="n"/>
       <c r="Q71" s="2189" t="n">
-        <v>2500</v>
+        <v>2700</v>
       </c>
       <c r="R71" s="2125">
         <f>K71/Q71</f>
         <v/>
       </c>
     </row>
-    <row r="72" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B72" s="2016" t="inlineStr">
-        <is>
-          <t>Musseletten:</t>
-        </is>
-      </c>
-      <c r="C72" s="2188" t="n"/>
-      <c r="D72" s="2160" t="n"/>
-      <c r="E72" s="2161" t="n"/>
-      <c r="F72" s="2161" t="n"/>
-      <c r="G72" s="2161" t="n"/>
-      <c r="H72" s="2161" t="n"/>
-      <c r="I72" s="2161" t="n"/>
-      <c r="J72" s="2170" t="n"/>
-      <c r="K72" s="2152">
-        <f>SUM(D72:I72)</f>
-        <v/>
-      </c>
+    <row r="72" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B72" s="1099" t="n"/>
+      <c r="C72" s="2170" t="n"/>
+      <c r="D72" s="1521" t="n"/>
+      <c r="E72" s="1521" t="n"/>
+      <c r="F72" s="1521" t="n"/>
+      <c r="G72" s="1521" t="n"/>
+      <c r="H72" s="1521" t="n"/>
+      <c r="I72" s="1521" t="n"/>
+      <c r="J72" s="1521" t="n"/>
+      <c r="K72" s="2190" t="n"/>
       <c r="L72" s="2112" t="n"/>
-      <c r="M72" s="2152">
-        <f>K72-SUM(K23:K24)*6--K25*12</f>
-        <v/>
-      </c>
+      <c r="M72" s="2177" t="n"/>
       <c r="N72" s="1521" t="n"/>
-      <c r="O72" s="1521" t="inlineStr">
-        <is>
-          <t>Doos á</t>
-        </is>
-      </c>
-      <c r="P72" s="1521" t="n"/>
-      <c r="Q72" s="2189" t="n">
-        <v>2700</v>
-      </c>
-      <c r="R72" s="2125">
-        <f>K72/Q72</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B73" s="1099" t="n"/>
-      <c r="C73" s="2170" t="n"/>
-      <c r="D73" s="1521" t="n"/>
-      <c r="E73" s="1521" t="n"/>
-      <c r="F73" s="1521" t="n"/>
-      <c r="G73" s="1521" t="n"/>
-      <c r="H73" s="1521" t="n"/>
-      <c r="I73" s="1521" t="n"/>
-      <c r="J73" s="1521" t="n"/>
-      <c r="K73" s="2190" t="n"/>
-      <c r="L73" s="2112" t="n"/>
-      <c r="M73" s="2177" t="n"/>
+      <c r="O72" s="2182">
+        <f>O62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B73" s="2172" t="inlineStr">
+        <is>
+          <t>VERBRUIKEN BLIK-artikelen</t>
+        </is>
+      </c>
+      <c r="C73" s="2147" t="inlineStr">
+        <is>
+          <t>Opmerkingen</t>
+        </is>
+      </c>
+      <c r="D73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="E73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="F73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="G73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="H73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="I73" s="2010" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="J73" s="2112" t="n"/>
+      <c r="K73" s="2010" t="inlineStr">
+        <is>
+          <t>TOTALEN</t>
+        </is>
+      </c>
+      <c r="L73" s="2191" t="n"/>
+      <c r="M73" s="2010" t="inlineStr">
+        <is>
+          <t>VERLIES</t>
+        </is>
+      </c>
       <c r="N73" s="1521" t="n"/>
-      <c r="O73" s="2182">
-        <f>O63</f>
-        <v/>
-      </c>
+      <c r="O73" s="2182" t="n"/>
+      <c r="P73" s="2182" t="n"/>
+      <c r="Q73" s="2182" t="n"/>
+      <c r="R73" s="2182" t="n"/>
     </row>
     <row r="74" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B74" s="2172" t="inlineStr">
-        <is>
-          <t>VERBRUIKEN BLIK-artikelen</t>
-        </is>
-      </c>
-      <c r="C74" s="2147" t="inlineStr">
-        <is>
-          <t>Opmerkingen</t>
-        </is>
-      </c>
-      <c r="D74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="E74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="F74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="G74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="H74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="I74" s="2010" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="J74" s="2112" t="n"/>
-      <c r="K74" s="2010" t="inlineStr">
-        <is>
-          <t>TOTALEN</t>
-        </is>
-      </c>
-      <c r="L74" s="2191" t="n"/>
-      <c r="M74" s="2010" t="inlineStr">
-        <is>
-          <t>VERLIES</t>
-        </is>
+      <c r="B74" s="2192" t="inlineStr">
+        <is>
+          <t>Blik 33cl</t>
+        </is>
+      </c>
+      <c r="C74" s="2176" t="n"/>
+      <c r="D74" s="2193" t="n"/>
+      <c r="E74" s="2194" t="n"/>
+      <c r="F74" s="2194" t="n"/>
+      <c r="G74" s="2194" t="n"/>
+      <c r="H74" s="2194" t="n"/>
+      <c r="I74" s="2194" t="n"/>
+      <c r="J74" s="1521" t="n"/>
+      <c r="K74" s="2152">
+        <f>SUM(D74:I74)</f>
+        <v/>
+      </c>
+      <c r="L74" s="2112" t="n"/>
+      <c r="M74" s="2177">
+        <f>K74-(K28*12)</f>
+        <v/>
       </c>
       <c r="N74" s="1521" t="n"/>
       <c r="O74" s="2182" t="n"/>
@@ -33136,24 +33141,21 @@
     <row r="75" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B75" s="2192" t="inlineStr">
         <is>
-          <t>Blik 33cl</t>
-        </is>
-      </c>
-      <c r="C75" s="2176" t="n"/>
-      <c r="D75" s="2193" t="n"/>
-      <c r="E75" s="2194" t="n"/>
-      <c r="F75" s="2194" t="n"/>
-      <c r="G75" s="2194" t="n"/>
-      <c r="H75" s="2194" t="n"/>
-      <c r="I75" s="2194" t="n"/>
+          <t>Blik 44cl</t>
+        </is>
+      </c>
+      <c r="C75" s="2195" t="n"/>
+      <c r="D75" s="2196" t="n"/>
+      <c r="E75" s="2197" t="n"/>
+      <c r="F75" s="2197" t="n"/>
+      <c r="G75" s="2197" t="n"/>
+      <c r="H75" s="2197" t="n"/>
+      <c r="I75" s="2197" t="n"/>
       <c r="J75" s="1521" t="n"/>
-      <c r="K75" s="2152">
-        <f>SUM(D75:I75)</f>
-        <v/>
-      </c>
+      <c r="K75" s="2152" t="n"/>
       <c r="L75" s="2112" t="n"/>
       <c r="M75" s="2177">
-        <f>K75-(K28*12)</f>
+        <f>K75-(K29*12)</f>
         <v/>
       </c>
       <c r="N75" s="1521" t="n"/>
@@ -33165,21 +33167,24 @@
     <row r="76" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B76" s="2192" t="inlineStr">
         <is>
-          <t>Blik 44cl</t>
-        </is>
-      </c>
-      <c r="C76" s="2195" t="n"/>
-      <c r="D76" s="2196" t="n"/>
-      <c r="E76" s="2197" t="n"/>
-      <c r="F76" s="2197" t="n"/>
-      <c r="G76" s="2197" t="n"/>
-      <c r="H76" s="2197" t="n"/>
-      <c r="I76" s="2197" t="n"/>
+          <t>Blik Deksel</t>
+        </is>
+      </c>
+      <c r="C76" s="1615" t="n"/>
+      <c r="D76" s="2167" t="n"/>
+      <c r="E76" s="2184" t="n"/>
+      <c r="F76" s="2184" t="n"/>
+      <c r="G76" s="2184" t="n"/>
+      <c r="H76" s="2184" t="n"/>
+      <c r="I76" s="2184" t="n"/>
       <c r="J76" s="1521" t="n"/>
-      <c r="K76" s="2152" t="n"/>
+      <c r="K76" s="2152">
+        <f>SUM(D76:I76)</f>
+        <v/>
+      </c>
       <c r="L76" s="2112" t="n"/>
       <c r="M76" s="2177">
-        <f>K76-(K29*12)</f>
+        <f>K76-(K28*12)</f>
         <v/>
       </c>
       <c r="N76" s="1521" t="n"/>
@@ -33191,7 +33196,7 @@
     <row r="77" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B77" s="2192" t="inlineStr">
         <is>
-          <t>Blik Deksel</t>
+          <t>Stickerlabel 33cl blik</t>
         </is>
       </c>
       <c r="C77" s="1615" t="n"/>
@@ -33220,7 +33225,7 @@
     <row r="78" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B78" s="2192" t="inlineStr">
         <is>
-          <t>Stickerlabel 33cl blik</t>
+          <t>Stickerlabel 44cl blik</t>
         </is>
       </c>
       <c r="C78" s="1615" t="n"/>
@@ -33231,13 +33236,10 @@
       <c r="H78" s="2184" t="n"/>
       <c r="I78" s="2184" t="n"/>
       <c r="J78" s="1521" t="n"/>
-      <c r="K78" s="2152">
-        <f>SUM(D78:I78)</f>
-        <v/>
-      </c>
+      <c r="K78" s="2152" t="n"/>
       <c r="L78" s="2112" t="n"/>
       <c r="M78" s="2177">
-        <f>K78-(K28*12)</f>
+        <f>K78-(K29*12)</f>
         <v/>
       </c>
       <c r="N78" s="1521" t="n"/>
@@ -33249,7 +33251,7 @@
     <row r="79" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B79" s="2192" t="inlineStr">
         <is>
-          <t>Stickerlabel 44cl blik</t>
+          <t>Omdozen 12x33cl blik - Blanco</t>
         </is>
       </c>
       <c r="C79" s="1615" t="n"/>
@@ -33260,10 +33262,13 @@
       <c r="H79" s="2184" t="n"/>
       <c r="I79" s="2184" t="n"/>
       <c r="J79" s="1521" t="n"/>
-      <c r="K79" s="2152" t="n"/>
+      <c r="K79" s="2152">
+        <f>SUM(D79:I79)</f>
+        <v/>
+      </c>
       <c r="L79" s="2112" t="n"/>
-      <c r="M79" s="2177">
-        <f>K79-(K29*12)</f>
+      <c r="M79" s="2152">
+        <f>K79-K28</f>
         <v/>
       </c>
       <c r="N79" s="1521" t="n"/>
@@ -33275,7 +33280,7 @@
     <row r="80" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B80" s="2192" t="inlineStr">
         <is>
-          <t>Omdozen 12x33cl blik - Blanco</t>
+          <t>Omdozen 24x33cl blik - Blanco</t>
         </is>
       </c>
       <c r="C80" s="1615" t="n"/>
@@ -33286,25 +33291,17 @@
       <c r="H80" s="2184" t="n"/>
       <c r="I80" s="2184" t="n"/>
       <c r="J80" s="1521" t="n"/>
-      <c r="K80" s="2152">
-        <f>SUM(D80:I80)</f>
-        <v/>
-      </c>
+      <c r="K80" s="2152" t="n"/>
       <c r="L80" s="2112" t="n"/>
       <c r="M80" s="2152">
-        <f>K80-K28</f>
-        <v/>
-      </c>
-      <c r="N80" s="1521" t="n"/>
-      <c r="O80" s="2182" t="n"/>
-      <c r="P80" s="2182" t="n"/>
-      <c r="Q80" s="2182" t="n"/>
-      <c r="R80" s="2182" t="n"/>
+        <f>K80-K29</f>
+        <v/>
+      </c>
     </row>
     <row r="81" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B81" s="2192" t="inlineStr">
         <is>
-          <t>Omdozen 24x33cl blik - Blanco</t>
+          <t>Omdozen 12x44cl blik - Blanco</t>
         </is>
       </c>
       <c r="C81" s="1615" t="n"/>
@@ -33318,14 +33315,14 @@
       <c r="K81" s="2152" t="n"/>
       <c r="L81" s="2112" t="n"/>
       <c r="M81" s="2152">
-        <f>K81-K29</f>
+        <f>K81-K30</f>
         <v/>
       </c>
     </row>
     <row r="82" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B82" s="2192" t="inlineStr">
         <is>
-          <t>Omdozen 12x44cl blik - Blanco</t>
+          <t>Omdozen 24x44cl blik - Blanco</t>
         </is>
       </c>
       <c r="C82" s="1615" t="n"/>
@@ -33339,112 +33336,115 @@
       <c r="K82" s="2152" t="n"/>
       <c r="L82" s="2112" t="n"/>
       <c r="M82" s="2152">
-        <f>K82-K30</f>
+        <f>K82-K31</f>
         <v/>
       </c>
     </row>
     <row r="83" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B83" s="2192" t="inlineStr">
-        <is>
-          <t>Omdozen 24x44cl blik - Blanco</t>
-        </is>
-      </c>
-      <c r="C83" s="1615" t="n"/>
-      <c r="D83" s="2167" t="n"/>
-      <c r="E83" s="2184" t="n"/>
-      <c r="F83" s="2184" t="n"/>
-      <c r="G83" s="2184" t="n"/>
-      <c r="H83" s="2184" t="n"/>
-      <c r="I83" s="2184" t="n"/>
+      <c r="B83" s="1099" t="n"/>
+      <c r="C83" s="2170" t="n"/>
+      <c r="D83" s="1521" t="n"/>
+      <c r="E83" s="1521" t="n"/>
+      <c r="F83" s="1521" t="n"/>
+      <c r="G83" s="1521" t="n"/>
+      <c r="H83" s="1521" t="n"/>
+      <c r="I83" s="1521" t="n"/>
       <c r="J83" s="1521" t="n"/>
-      <c r="K83" s="2152" t="n"/>
+      <c r="K83" s="2190" t="n"/>
       <c r="L83" s="2112" t="n"/>
-      <c r="M83" s="2152">
-        <f>K83-K31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B84" s="1099" t="n"/>
-      <c r="C84" s="2170" t="n"/>
-      <c r="D84" s="1521" t="n"/>
-      <c r="E84" s="1521" t="n"/>
-      <c r="F84" s="1521" t="n"/>
-      <c r="G84" s="1521" t="n"/>
-      <c r="H84" s="1521" t="n"/>
-      <c r="I84" s="1521" t="n"/>
-      <c r="J84" s="1521" t="n"/>
-      <c r="K84" s="2190" t="n"/>
-      <c r="L84" s="2112" t="n"/>
-      <c r="M84" s="2177" t="n"/>
-    </row>
-    <row r="85" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B85" s="2172" t="inlineStr">
+      <c r="M83" s="2177" t="n"/>
+    </row>
+    <row r="84" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B84" s="2172" t="inlineStr">
         <is>
           <t>VERBRUIKEN FUST-artikelen</t>
         </is>
       </c>
-      <c r="C85" s="2147" t="inlineStr">
+      <c r="C84" s="2147" t="inlineStr">
         <is>
           <t>Opmerkingen</t>
         </is>
       </c>
-      <c r="D85" s="2010" t="inlineStr">
+      <c r="D84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="E85" s="2010" t="inlineStr">
+      <c r="E84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="F85" s="2010" t="inlineStr">
+      <c r="F84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="G85" s="2010" t="inlineStr">
+      <c r="G84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="H85" s="2010" t="inlineStr">
+      <c r="H84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="I85" s="2010" t="inlineStr">
+      <c r="I84" s="2010" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="J85" s="2112" t="n"/>
-      <c r="K85" s="2010" t="inlineStr">
+      <c r="J84" s="2112" t="n"/>
+      <c r="K84" s="2010" t="inlineStr">
         <is>
           <t>TOTALEN</t>
         </is>
       </c>
-      <c r="L85" s="2191" t="n"/>
-      <c r="M85" s="2010" t="inlineStr">
+      <c r="L84" s="2191" t="n"/>
+      <c r="M84" s="2010" t="inlineStr">
         <is>
           <t>VERLIES</t>
         </is>
+      </c>
+    </row>
+    <row r="85" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B85" s="2016" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global Keg 20L: </t>
+        </is>
+      </c>
+      <c r="C85" s="2176" t="n"/>
+      <c r="D85" s="2193" t="n"/>
+      <c r="E85" s="2194" t="n"/>
+      <c r="F85" s="2194" t="n"/>
+      <c r="G85" s="2194" t="n"/>
+      <c r="H85" s="2194" t="n"/>
+      <c r="I85" s="2194" t="n"/>
+      <c r="J85" s="1521" t="n"/>
+      <c r="K85" s="2152">
+        <f>SUM(D85:I85)</f>
+        <v/>
+      </c>
+      <c r="L85" s="2112" t="n"/>
+      <c r="M85" s="2152">
+        <f>K85-K34</f>
+        <v/>
       </c>
     </row>
     <row r="86" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B86" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global Keg 20L: </t>
-        </is>
-      </c>
-      <c r="C86" s="2176" t="n"/>
-      <c r="D86" s="2193" t="n"/>
-      <c r="E86" s="2194" t="n"/>
-      <c r="F86" s="2194" t="n"/>
-      <c r="G86" s="2194" t="n"/>
-      <c r="H86" s="2194" t="n"/>
-      <c r="I86" s="2194" t="n"/>
+          <t xml:space="preserve">Jopen Fust 20L: </t>
+        </is>
+      </c>
+      <c r="C86" s="1615" t="n"/>
+      <c r="D86" s="2167" t="n"/>
+      <c r="E86" s="2184" t="n"/>
+      <c r="F86" s="2184" t="n"/>
+      <c r="G86" s="2184" t="n"/>
+      <c r="H86" s="2184" t="n"/>
+      <c r="I86" s="2184" t="n"/>
       <c r="J86" s="1521" t="n"/>
       <c r="K86" s="2152">
         <f>SUM(D86:I86)</f>
@@ -33452,14 +33452,14 @@
       </c>
       <c r="L86" s="2112" t="n"/>
       <c r="M86" s="2152">
-        <f>K86-K34</f>
+        <f>K86-K35</f>
         <v/>
       </c>
     </row>
     <row r="87" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B87" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 20L: </t>
+          <t xml:space="preserve">Jopen Fust 30L: </t>
         </is>
       </c>
       <c r="C87" s="1615" t="n"/>
@@ -33469,21 +33469,21 @@
       <c r="G87" s="2184" t="n"/>
       <c r="H87" s="2184" t="n"/>
       <c r="I87" s="2184" t="n"/>
-      <c r="J87" s="1521" t="n"/>
+      <c r="J87" s="2170" t="n"/>
       <c r="K87" s="2152">
         <f>SUM(D87:I87)</f>
         <v/>
       </c>
       <c r="L87" s="2112" t="n"/>
       <c r="M87" s="2152">
-        <f>K87-K35</f>
+        <f>K87-K36</f>
         <v/>
       </c>
     </row>
     <row r="88" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B88" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 30L: </t>
+          <t xml:space="preserve">Jopen Fust 50L: </t>
         </is>
       </c>
       <c r="C88" s="1615" t="n"/>
@@ -33493,106 +33493,106 @@
       <c r="G88" s="2184" t="n"/>
       <c r="H88" s="2184" t="n"/>
       <c r="I88" s="2184" t="n"/>
-      <c r="J88" s="2170" t="n"/>
+      <c r="J88" s="1521" t="n"/>
       <c r="K88" s="2152">
         <f>SUM(D88:I88)</f>
         <v/>
       </c>
       <c r="L88" s="2112" t="n"/>
       <c r="M88" s="2152">
-        <f>K88-K36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B89" s="2016" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jopen Fust 50L: </t>
-        </is>
-      </c>
-      <c r="C89" s="1615" t="n"/>
-      <c r="D89" s="2167" t="n"/>
-      <c r="E89" s="2184" t="n"/>
-      <c r="F89" s="2184" t="n"/>
-      <c r="G89" s="2184" t="n"/>
-      <c r="H89" s="2184" t="n"/>
-      <c r="I89" s="2184" t="n"/>
+        <f>K88-K37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B89" s="2185" t="n"/>
+      <c r="C89" s="2198" t="n"/>
+      <c r="D89" s="2156" t="n"/>
+      <c r="E89" s="2156" t="n"/>
+      <c r="F89" s="2156" t="n"/>
+      <c r="G89" s="2156" t="n"/>
+      <c r="H89" s="2156" t="n"/>
+      <c r="I89" s="2156" t="n"/>
       <c r="J89" s="1521" t="n"/>
-      <c r="K89" s="2152">
-        <f>SUM(D89:I89)</f>
-        <v/>
-      </c>
+      <c r="K89" s="2152" t="n"/>
       <c r="L89" s="2112" t="n"/>
-      <c r="M89" s="2152">
-        <f>K89-K37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B90" s="2185" t="n"/>
-      <c r="C90" s="2198" t="n"/>
-      <c r="D90" s="2156" t="n"/>
-      <c r="E90" s="2156" t="n"/>
-      <c r="F90" s="2156" t="n"/>
-      <c r="G90" s="2156" t="n"/>
-      <c r="H90" s="2156" t="n"/>
-      <c r="I90" s="2156" t="n"/>
+      <c r="M89" s="2152" t="n"/>
+    </row>
+    <row r="90" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B90" s="2016" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fustdop: </t>
+        </is>
+      </c>
+      <c r="C90" s="1615" t="n"/>
+      <c r="D90" s="2167" t="n"/>
+      <c r="E90" s="2184" t="n"/>
+      <c r="F90" s="2184" t="n"/>
+      <c r="G90" s="2184" t="n"/>
+      <c r="H90" s="2184" t="n"/>
+      <c r="I90" s="2184" t="n"/>
       <c r="J90" s="1521" t="n"/>
-      <c r="K90" s="2152" t="n"/>
+      <c r="K90" s="2152">
+        <f>SUM(D90:I90)</f>
+        <v/>
+      </c>
       <c r="L90" s="2112" t="n"/>
-      <c r="M90" s="2152" t="n"/>
-    </row>
-    <row r="91" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B91" s="2016" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fustdop: </t>
-        </is>
-      </c>
-      <c r="C91" s="1615" t="n"/>
-      <c r="D91" s="2167" t="n"/>
-      <c r="E91" s="2184" t="n"/>
-      <c r="F91" s="2184" t="n"/>
-      <c r="G91" s="2184" t="n"/>
-      <c r="H91" s="2184" t="n"/>
-      <c r="I91" s="2184" t="n"/>
-      <c r="J91" s="1521" t="n"/>
-      <c r="K91" s="2152">
-        <f>SUM(D91:I91)</f>
-        <v/>
-      </c>
+      <c r="M90" s="2152">
+        <f>K90-SUM(K34:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B91" s="1099" t="n"/>
+      <c r="C91" s="2170" t="n"/>
+      <c r="D91" s="1521" t="n"/>
+      <c r="E91" s="1521" t="n"/>
+      <c r="F91" s="1521" t="n"/>
+      <c r="G91" s="1521" t="n"/>
+      <c r="H91" s="1521" t="n"/>
+      <c r="I91" s="1521" t="n"/>
+      <c r="J91" s="2170" t="n"/>
+      <c r="K91" s="2152" t="n"/>
       <c r="L91" s="2112" t="n"/>
-      <c r="M91" s="2152">
-        <f>K91-SUM(K34:K37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B92" s="1099" t="n"/>
-      <c r="C92" s="2170" t="n"/>
-      <c r="D92" s="1521" t="n"/>
-      <c r="E92" s="1521" t="n"/>
-      <c r="F92" s="1521" t="n"/>
-      <c r="G92" s="1521" t="n"/>
-      <c r="H92" s="1521" t="n"/>
-      <c r="I92" s="1521" t="n"/>
-      <c r="J92" s="2170" t="n"/>
-      <c r="K92" s="2152" t="n"/>
+      <c r="M91" s="2152" t="n"/>
+    </row>
+    <row r="92" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B92" s="2199" t="inlineStr">
+        <is>
+          <t>KeyKegFustdop:</t>
+        </is>
+      </c>
+      <c r="C92" s="2179" t="n"/>
+      <c r="D92" s="2193" t="n"/>
+      <c r="E92" s="2194" t="n"/>
+      <c r="F92" s="2194" t="n"/>
+      <c r="G92" s="2194" t="n"/>
+      <c r="H92" s="2194" t="n"/>
+      <c r="I92" s="2194" t="n"/>
+      <c r="J92" s="1521" t="n"/>
+      <c r="K92" s="2152">
+        <f>SUM(D92:I92)</f>
+        <v/>
+      </c>
       <c r="L92" s="2112" t="n"/>
-      <c r="M92" s="2152" t="n"/>
+      <c r="M92" s="2152">
+        <f>K92-K34-K41</f>
+        <v/>
+      </c>
     </row>
     <row r="93" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B93" s="2199" t="inlineStr">
-        <is>
-          <t>KeyKegFustdop:</t>
-        </is>
-      </c>
-      <c r="C93" s="2179" t="n"/>
-      <c r="D93" s="2193" t="n"/>
-      <c r="E93" s="2194" t="n"/>
-      <c r="F93" s="2194" t="n"/>
-      <c r="G93" s="2194" t="n"/>
-      <c r="H93" s="2194" t="n"/>
-      <c r="I93" s="2194" t="n"/>
+      <c r="B93" s="2200" t="inlineStr">
+        <is>
+          <t>KeyKeg 20L - Leeg</t>
+        </is>
+      </c>
+      <c r="C93" s="2201" t="n"/>
+      <c r="D93" s="2202" t="n"/>
+      <c r="E93" s="2203" t="n"/>
+      <c r="F93" s="2203" t="n"/>
+      <c r="G93" s="2203" t="n"/>
+      <c r="H93" s="2203" t="n"/>
+      <c r="I93" s="2203" t="n"/>
       <c r="J93" s="1521" t="n"/>
       <c r="K93" s="2152">
         <f>SUM(D93:I93)</f>
@@ -33600,23 +33600,23 @@
       </c>
       <c r="L93" s="2112" t="n"/>
       <c r="M93" s="2152">
-        <f>K93-K34-K42</f>
+        <f>K93-K34</f>
         <v/>
       </c>
     </row>
     <row r="94" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B94" s="2200" t="inlineStr">
-        <is>
-          <t>KeyKeg 20L - Leeg</t>
-        </is>
-      </c>
-      <c r="C94" s="2201" t="n"/>
-      <c r="D94" s="2202" t="n"/>
-      <c r="E94" s="2203" t="n"/>
-      <c r="F94" s="2203" t="n"/>
-      <c r="G94" s="2203" t="n"/>
-      <c r="H94" s="2203" t="n"/>
-      <c r="I94" s="2203" t="n"/>
+      <c r="B94" s="2016" t="inlineStr">
+        <is>
+          <t>KeyKeg 30L - Leeg</t>
+        </is>
+      </c>
+      <c r="C94" s="2204" t="n"/>
+      <c r="D94" s="2160" t="n"/>
+      <c r="E94" s="2161" t="n"/>
+      <c r="F94" s="2161" t="n"/>
+      <c r="G94" s="2161" t="n"/>
+      <c r="H94" s="2161" t="n"/>
+      <c r="I94" s="2161" t="n"/>
       <c r="J94" s="1521" t="n"/>
       <c r="K94" s="2152">
         <f>SUM(D94:I94)</f>
@@ -33624,64 +33624,48 @@
       </c>
       <c r="L94" s="2112" t="n"/>
       <c r="M94" s="2152">
-        <f>K94-K34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B95" s="2016" t="inlineStr">
-        <is>
-          <t>KeyKeg 30L - Leeg</t>
-        </is>
-      </c>
-      <c r="C95" s="2204" t="n"/>
-      <c r="D95" s="2160" t="n"/>
-      <c r="E95" s="2161" t="n"/>
-      <c r="F95" s="2161" t="n"/>
-      <c r="G95" s="2161" t="n"/>
-      <c r="H95" s="2161" t="n"/>
-      <c r="I95" s="2161" t="n"/>
-      <c r="J95" s="1521" t="n"/>
-      <c r="K95" s="2152">
-        <f>SUM(D95:I95)</f>
-        <v/>
-      </c>
-      <c r="L95" s="2112" t="n"/>
-      <c r="M95" s="2152">
-        <f>K95-K42</f>
-        <v/>
-      </c>
-    </row>
+        <f>K94-K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="15" customHeight="1" s="1339"/>
     <row r="96" ht="15" customHeight="1" s="1339"/>
-    <row r="97" ht="15" customHeight="1" s="1339"/>
+    <row r="97" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B97" s="2013" t="inlineStr">
+        <is>
+          <t>Ingevoerd in Mdrank</t>
+        </is>
+      </c>
+      <c r="C97" s="2026" t="inlineStr">
+        <is>
+          <t>door:</t>
+        </is>
+      </c>
+      <c r="D97" s="2205" t="n"/>
+      <c r="E97" s="1115" t="n"/>
+    </row>
     <row r="98" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B98" s="2013" t="inlineStr">
-        <is>
-          <t>Ingevoerd in Mdrank</t>
-        </is>
-      </c>
+      <c r="B98" s="2206" t="n"/>
       <c r="C98" s="2026" t="inlineStr">
         <is>
-          <t>door:</t>
-        </is>
-      </c>
-      <c r="D98" s="2205" t="n"/>
+          <t>datum:</t>
+        </is>
+      </c>
+      <c r="D98" s="2215" t="n"/>
       <c r="E98" s="1115" t="n"/>
     </row>
     <row r="99" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B99" s="2206" t="n"/>
-      <c r="C99" s="2026" t="inlineStr">
-        <is>
-          <t>datum:</t>
-        </is>
-      </c>
-      <c r="D99" s="2215" t="n"/>
-      <c r="E99" s="1115" t="n"/>
+      <c r="B99" s="2208" t="inlineStr">
+        <is>
+          <t>V2,1 : 09-10-17 KYT</t>
+        </is>
+      </c>
+      <c r="C99" s="1521" t="n"/>
     </row>
     <row r="100" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B100" s="2208" t="inlineStr">
         <is>
-          <t>V2,1 : 09-10-17 KYT</t>
+          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
         </is>
       </c>
       <c r="C100" s="1521" t="n"/>
@@ -33689,7 +33673,7 @@
     <row r="101" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B101" s="2208" t="inlineStr">
         <is>
-          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
+          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
         </is>
       </c>
       <c r="C101" s="1521" t="n"/>
@@ -33697,54 +33681,46 @@
     <row r="102" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B102" s="2208" t="inlineStr">
         <is>
-          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
+          <t>v3 6/2/24 TW</t>
         </is>
       </c>
       <c r="C102" s="1521" t="n"/>
-    </row>
-    <row r="103" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B103" s="2208" t="inlineStr">
-        <is>
-          <t>v3 6/2/24 TW</t>
-        </is>
-      </c>
-      <c r="C103" s="1521" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
     <mergeCell ref="M11:O11"/>
     <mergeCell ref="M10:O10"/>
     <mergeCell ref="M3:M5"/>
-    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="K43:M43"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B1:I2"/>
-    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="D98:E98"/>
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="C3:E4"/>
-    <mergeCell ref="O73:R73"/>
+    <mergeCell ref="O72:R72"/>
     <mergeCell ref="M12:O12"/>
     <mergeCell ref="Q8:R8"/>
     <mergeCell ref="H3:I4"/>
     <mergeCell ref="M8:O8"/>
     <mergeCell ref="B6:C11"/>
     <mergeCell ref="Q3:R4"/>
-    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="K48:M48"/>
     <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B48:I48"/>
     <mergeCell ref="K15:M15"/>
-    <mergeCell ref="O63:R63"/>
+    <mergeCell ref="O62:R62"/>
     <mergeCell ref="F3:G4"/>
-    <mergeCell ref="D98:E98"/>
+    <mergeCell ref="D97:E97"/>
     <mergeCell ref="M9:O9"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="M1:R1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M45:M46">
+  <conditionalFormatting sqref="M44:M45">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="29" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M62">
+  <conditionalFormatting sqref="M61">
     <cfRule type="cellIs" rank="0" priority="3" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33765,37 +33741,37 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K80:K83">
+  <conditionalFormatting sqref="K79:K82">
     <cfRule type="cellIs" rank="0" priority="8" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="33" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K78:K79">
+  <conditionalFormatting sqref="K77:K78">
     <cfRule type="cellIs" rank="0" priority="9" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="33" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K77">
+  <conditionalFormatting sqref="K76">
     <cfRule type="cellIs" rank="0" priority="10" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="33" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K75:K76">
+  <conditionalFormatting sqref="K74:K75">
     <cfRule type="cellIs" rank="0" priority="11" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="33" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M74">
+  <conditionalFormatting sqref="M73">
     <cfRule type="cellIs" rank="0" priority="12" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K74">
+  <conditionalFormatting sqref="K73">
     <cfRule type="cellIs" rank="0" priority="13" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M75:M83">
+  <conditionalFormatting sqref="M74:M82">
     <cfRule type="cellIs" rank="0" priority="14" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33806,7 +33782,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M87">
+  <conditionalFormatting sqref="M86">
     <cfRule type="cellIs" rank="0" priority="17" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33817,12 +33793,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K87">
+  <conditionalFormatting sqref="K86">
     <cfRule type="cellIs" rank="0" priority="20" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M88">
+  <conditionalFormatting sqref="M87">
     <cfRule type="cellIs" rank="0" priority="21" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33833,12 +33809,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K88">
+  <conditionalFormatting sqref="K87">
     <cfRule type="cellIs" rank="0" priority="24" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M89:M90">
+  <conditionalFormatting sqref="M88:M89">
     <cfRule type="cellIs" rank="0" priority="25" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33849,7 +33825,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K89:K90">
+  <conditionalFormatting sqref="K88:K89">
     <cfRule type="cellIs" rank="0" priority="28" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33859,7 +33835,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M86">
+  <conditionalFormatting sqref="M85">
     <cfRule type="cellIs" rank="0" priority="30" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33870,22 +33846,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K86">
+  <conditionalFormatting sqref="K85">
     <cfRule type="cellIs" rank="0" priority="33" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M85">
+  <conditionalFormatting sqref="M84">
     <cfRule type="cellIs" rank="0" priority="34" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M34 M36:M42">
+  <conditionalFormatting sqref="M34 M36:M41">
     <cfRule type="cellIs" rank="0" priority="35" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="29" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M51:M61 M63:M73 M84 M91:M96">
+  <conditionalFormatting sqref="M50:M60 M62:M72 M83 M90:M95">
     <cfRule type="cellIs" rank="0" priority="36" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33901,17 +33877,17 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K85">
+  <conditionalFormatting sqref="K84">
     <cfRule type="cellIs" rank="0" priority="40" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K51:K54 K56:K57 K59:K60 K64:K66 K68:K70">
+  <conditionalFormatting sqref="K50:K53 K55:K56 K58:K59 K63:K65 K67:K69">
     <cfRule type="cellIs" rank="0" priority="41" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="33" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K42 K45:K47 K91:K96 R62 R71:R72">
+  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K41 K44:K46 K90:K95 R61 R70:R71">
     <cfRule type="cellIs" rank="0" priority="42" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Afvulverslag: verbruiksrij 'Global Keg 20L' verwijderd
- Rij 85 (VERBRUIKEN FUST-artikelen) weg, alles eronder 1 rij omhoog
- Afvullen!C61 telt nu SUM(Afvulverslag!M85:M86) (Jopen Fust 20L + 30L verlies)
- Bijbehorende conditional formatting-regels opgeruimd
- fix-american-dates.js: Afvulverslag!D98 -> D97

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CvHodB7rajqHXKYMVFnfMs
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -29784,7 +29784,7 @@
       </c>
       <c r="B61" s="2069" t="n"/>
       <c r="C61" s="2078">
-        <f>SUM(Afvulverslag!M85:M87)</f>
+        <f>SUM(Afvulverslag!M85:M86)</f>
         <v/>
       </c>
       <c r="D61" s="2070" t="n"/>
@@ -31093,7 +31093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R102"/>
+  <dimension ref="A1:R101"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.00390625" defaultRowHeight="15" zeroHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="2.5" customWidth="1" style="2094" min="1" max="1"/>
@@ -33411,16 +33411,16 @@
     <row r="85" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B85" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global Keg 20L: </t>
-        </is>
-      </c>
-      <c r="C85" s="2176" t="n"/>
-      <c r="D85" s="2193" t="n"/>
-      <c r="E85" s="2194" t="n"/>
-      <c r="F85" s="2194" t="n"/>
-      <c r="G85" s="2194" t="n"/>
-      <c r="H85" s="2194" t="n"/>
-      <c r="I85" s="2194" t="n"/>
+          <t xml:space="preserve">Jopen Fust 20L: </t>
+        </is>
+      </c>
+      <c r="C85" s="1615" t="n"/>
+      <c r="D85" s="2167" t="n"/>
+      <c r="E85" s="2184" t="n"/>
+      <c r="F85" s="2184" t="n"/>
+      <c r="G85" s="2184" t="n"/>
+      <c r="H85" s="2184" t="n"/>
+      <c r="I85" s="2184" t="n"/>
       <c r="J85" s="1521" t="n"/>
       <c r="K85" s="2152">
         <f>SUM(D85:I85)</f>
@@ -33428,14 +33428,14 @@
       </c>
       <c r="L85" s="2112" t="n"/>
       <c r="M85" s="2152">
-        <f>K85-K34</f>
+        <f>K85-K35</f>
         <v/>
       </c>
     </row>
     <row r="86" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B86" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 20L: </t>
+          <t xml:space="preserve">Jopen Fust 30L: </t>
         </is>
       </c>
       <c r="C86" s="1615" t="n"/>
@@ -33445,21 +33445,21 @@
       <c r="G86" s="2184" t="n"/>
       <c r="H86" s="2184" t="n"/>
       <c r="I86" s="2184" t="n"/>
-      <c r="J86" s="1521" t="n"/>
+      <c r="J86" s="2170" t="n"/>
       <c r="K86" s="2152">
         <f>SUM(D86:I86)</f>
         <v/>
       </c>
       <c r="L86" s="2112" t="n"/>
       <c r="M86" s="2152">
-        <f>K86-K35</f>
+        <f>K86-K36</f>
         <v/>
       </c>
     </row>
     <row r="87" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B87" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 30L: </t>
+          <t xml:space="preserve">Jopen Fust 50L: </t>
         </is>
       </c>
       <c r="C87" s="1615" t="n"/>
@@ -33469,106 +33469,106 @@
       <c r="G87" s="2184" t="n"/>
       <c r="H87" s="2184" t="n"/>
       <c r="I87" s="2184" t="n"/>
-      <c r="J87" s="2170" t="n"/>
+      <c r="J87" s="1521" t="n"/>
       <c r="K87" s="2152">
         <f>SUM(D87:I87)</f>
         <v/>
       </c>
       <c r="L87" s="2112" t="n"/>
       <c r="M87" s="2152">
-        <f>K87-K36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B88" s="2016" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jopen Fust 50L: </t>
-        </is>
-      </c>
-      <c r="C88" s="1615" t="n"/>
-      <c r="D88" s="2167" t="n"/>
-      <c r="E88" s="2184" t="n"/>
-      <c r="F88" s="2184" t="n"/>
-      <c r="G88" s="2184" t="n"/>
-      <c r="H88" s="2184" t="n"/>
-      <c r="I88" s="2184" t="n"/>
+        <f>K87-K37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B88" s="2185" t="n"/>
+      <c r="C88" s="2198" t="n"/>
+      <c r="D88" s="2156" t="n"/>
+      <c r="E88" s="2156" t="n"/>
+      <c r="F88" s="2156" t="n"/>
+      <c r="G88" s="2156" t="n"/>
+      <c r="H88" s="2156" t="n"/>
+      <c r="I88" s="2156" t="n"/>
       <c r="J88" s="1521" t="n"/>
-      <c r="K88" s="2152">
-        <f>SUM(D88:I88)</f>
-        <v/>
-      </c>
+      <c r="K88" s="2152" t="n"/>
       <c r="L88" s="2112" t="n"/>
-      <c r="M88" s="2152">
-        <f>K88-K37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B89" s="2185" t="n"/>
-      <c r="C89" s="2198" t="n"/>
-      <c r="D89" s="2156" t="n"/>
-      <c r="E89" s="2156" t="n"/>
-      <c r="F89" s="2156" t="n"/>
-      <c r="G89" s="2156" t="n"/>
-      <c r="H89" s="2156" t="n"/>
-      <c r="I89" s="2156" t="n"/>
+      <c r="M88" s="2152" t="n"/>
+    </row>
+    <row r="89" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B89" s="2016" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fustdop: </t>
+        </is>
+      </c>
+      <c r="C89" s="1615" t="n"/>
+      <c r="D89" s="2167" t="n"/>
+      <c r="E89" s="2184" t="n"/>
+      <c r="F89" s="2184" t="n"/>
+      <c r="G89" s="2184" t="n"/>
+      <c r="H89" s="2184" t="n"/>
+      <c r="I89" s="2184" t="n"/>
       <c r="J89" s="1521" t="n"/>
-      <c r="K89" s="2152" t="n"/>
+      <c r="K89" s="2152">
+        <f>SUM(D89:I89)</f>
+        <v/>
+      </c>
       <c r="L89" s="2112" t="n"/>
-      <c r="M89" s="2152" t="n"/>
-    </row>
-    <row r="90" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B90" s="2016" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fustdop: </t>
-        </is>
-      </c>
-      <c r="C90" s="1615" t="n"/>
-      <c r="D90" s="2167" t="n"/>
-      <c r="E90" s="2184" t="n"/>
-      <c r="F90" s="2184" t="n"/>
-      <c r="G90" s="2184" t="n"/>
-      <c r="H90" s="2184" t="n"/>
-      <c r="I90" s="2184" t="n"/>
-      <c r="J90" s="1521" t="n"/>
-      <c r="K90" s="2152">
-        <f>SUM(D90:I90)</f>
-        <v/>
-      </c>
+      <c r="M89" s="2152">
+        <f>K89-SUM(K34:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B90" s="1099" t="n"/>
+      <c r="C90" s="2170" t="n"/>
+      <c r="D90" s="1521" t="n"/>
+      <c r="E90" s="1521" t="n"/>
+      <c r="F90" s="1521" t="n"/>
+      <c r="G90" s="1521" t="n"/>
+      <c r="H90" s="1521" t="n"/>
+      <c r="I90" s="1521" t="n"/>
+      <c r="J90" s="2170" t="n"/>
+      <c r="K90" s="2152" t="n"/>
       <c r="L90" s="2112" t="n"/>
-      <c r="M90" s="2152">
-        <f>K90-SUM(K34:K37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B91" s="1099" t="n"/>
-      <c r="C91" s="2170" t="n"/>
-      <c r="D91" s="1521" t="n"/>
-      <c r="E91" s="1521" t="n"/>
-      <c r="F91" s="1521" t="n"/>
-      <c r="G91" s="1521" t="n"/>
-      <c r="H91" s="1521" t="n"/>
-      <c r="I91" s="1521" t="n"/>
-      <c r="J91" s="2170" t="n"/>
-      <c r="K91" s="2152" t="n"/>
+      <c r="M90" s="2152" t="n"/>
+    </row>
+    <row r="91" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B91" s="2199" t="inlineStr">
+        <is>
+          <t>KeyKegFustdop:</t>
+        </is>
+      </c>
+      <c r="C91" s="2179" t="n"/>
+      <c r="D91" s="2193" t="n"/>
+      <c r="E91" s="2194" t="n"/>
+      <c r="F91" s="2194" t="n"/>
+      <c r="G91" s="2194" t="n"/>
+      <c r="H91" s="2194" t="n"/>
+      <c r="I91" s="2194" t="n"/>
+      <c r="J91" s="1521" t="n"/>
+      <c r="K91" s="2152">
+        <f>SUM(D91:I91)</f>
+        <v/>
+      </c>
       <c r="L91" s="2112" t="n"/>
-      <c r="M91" s="2152" t="n"/>
+      <c r="M91" s="2152">
+        <f>K91-K34-K41</f>
+        <v/>
+      </c>
     </row>
     <row r="92" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B92" s="2199" t="inlineStr">
-        <is>
-          <t>KeyKegFustdop:</t>
-        </is>
-      </c>
-      <c r="C92" s="2179" t="n"/>
-      <c r="D92" s="2193" t="n"/>
-      <c r="E92" s="2194" t="n"/>
-      <c r="F92" s="2194" t="n"/>
-      <c r="G92" s="2194" t="n"/>
-      <c r="H92" s="2194" t="n"/>
-      <c r="I92" s="2194" t="n"/>
+      <c r="B92" s="2200" t="inlineStr">
+        <is>
+          <t>KeyKeg 20L - Leeg</t>
+        </is>
+      </c>
+      <c r="C92" s="2201" t="n"/>
+      <c r="D92" s="2202" t="n"/>
+      <c r="E92" s="2203" t="n"/>
+      <c r="F92" s="2203" t="n"/>
+      <c r="G92" s="2203" t="n"/>
+      <c r="H92" s="2203" t="n"/>
+      <c r="I92" s="2203" t="n"/>
       <c r="J92" s="1521" t="n"/>
       <c r="K92" s="2152">
         <f>SUM(D92:I92)</f>
@@ -33576,23 +33576,23 @@
       </c>
       <c r="L92" s="2112" t="n"/>
       <c r="M92" s="2152">
-        <f>K92-K34-K41</f>
+        <f>K92-K34</f>
         <v/>
       </c>
     </row>
     <row r="93" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B93" s="2200" t="inlineStr">
-        <is>
-          <t>KeyKeg 20L - Leeg</t>
-        </is>
-      </c>
-      <c r="C93" s="2201" t="n"/>
-      <c r="D93" s="2202" t="n"/>
-      <c r="E93" s="2203" t="n"/>
-      <c r="F93" s="2203" t="n"/>
-      <c r="G93" s="2203" t="n"/>
-      <c r="H93" s="2203" t="n"/>
-      <c r="I93" s="2203" t="n"/>
+      <c r="B93" s="2016" t="inlineStr">
+        <is>
+          <t>KeyKeg 30L - Leeg</t>
+        </is>
+      </c>
+      <c r="C93" s="2204" t="n"/>
+      <c r="D93" s="2160" t="n"/>
+      <c r="E93" s="2161" t="n"/>
+      <c r="F93" s="2161" t="n"/>
+      <c r="G93" s="2161" t="n"/>
+      <c r="H93" s="2161" t="n"/>
+      <c r="I93" s="2161" t="n"/>
       <c r="J93" s="1521" t="n"/>
       <c r="K93" s="2152">
         <f>SUM(D93:I93)</f>
@@ -33600,64 +33600,48 @@
       </c>
       <c r="L93" s="2112" t="n"/>
       <c r="M93" s="2152">
-        <f>K93-K34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B94" s="2016" t="inlineStr">
-        <is>
-          <t>KeyKeg 30L - Leeg</t>
-        </is>
-      </c>
-      <c r="C94" s="2204" t="n"/>
-      <c r="D94" s="2160" t="n"/>
-      <c r="E94" s="2161" t="n"/>
-      <c r="F94" s="2161" t="n"/>
-      <c r="G94" s="2161" t="n"/>
-      <c r="H94" s="2161" t="n"/>
-      <c r="I94" s="2161" t="n"/>
-      <c r="J94" s="1521" t="n"/>
-      <c r="K94" s="2152">
-        <f>SUM(D94:I94)</f>
-        <v/>
-      </c>
-      <c r="L94" s="2112" t="n"/>
-      <c r="M94" s="2152">
-        <f>K94-K41</f>
-        <v/>
-      </c>
-    </row>
+        <f>K93-K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" ht="15" customHeight="1" s="1339"/>
     <row r="95" ht="15" customHeight="1" s="1339"/>
-    <row r="96" ht="15" customHeight="1" s="1339"/>
+    <row r="96" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B96" s="2013" t="inlineStr">
+        <is>
+          <t>Ingevoerd in Mdrank</t>
+        </is>
+      </c>
+      <c r="C96" s="2026" t="inlineStr">
+        <is>
+          <t>door:</t>
+        </is>
+      </c>
+      <c r="D96" s="2205" t="n"/>
+      <c r="E96" s="1115" t="n"/>
+    </row>
     <row r="97" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B97" s="2013" t="inlineStr">
-        <is>
-          <t>Ingevoerd in Mdrank</t>
-        </is>
-      </c>
+      <c r="B97" s="2206" t="n"/>
       <c r="C97" s="2026" t="inlineStr">
         <is>
-          <t>door:</t>
-        </is>
-      </c>
-      <c r="D97" s="2205" t="n"/>
+          <t>datum:</t>
+        </is>
+      </c>
+      <c r="D97" s="2215" t="n"/>
       <c r="E97" s="1115" t="n"/>
     </row>
     <row r="98" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B98" s="2206" t="n"/>
-      <c r="C98" s="2026" t="inlineStr">
-        <is>
-          <t>datum:</t>
-        </is>
-      </c>
-      <c r="D98" s="2215" t="n"/>
-      <c r="E98" s="1115" t="n"/>
+      <c r="B98" s="2208" t="inlineStr">
+        <is>
+          <t>V2,1 : 09-10-17 KYT</t>
+        </is>
+      </c>
+      <c r="C98" s="1521" t="n"/>
     </row>
     <row r="99" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B99" s="2208" t="inlineStr">
         <is>
-          <t>V2,1 : 09-10-17 KYT</t>
+          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
         </is>
       </c>
       <c r="C99" s="1521" t="n"/>
@@ -33665,7 +33649,7 @@
     <row r="100" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B100" s="2208" t="inlineStr">
         <is>
-          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
+          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
         </is>
       </c>
       <c r="C100" s="1521" t="n"/>
@@ -33673,18 +33657,10 @@
     <row r="101" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B101" s="2208" t="inlineStr">
         <is>
-          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
+          <t>v3 6/2/24 TW</t>
         </is>
       </c>
       <c r="C101" s="1521" t="n"/>
-    </row>
-    <row r="102" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B102" s="2208" t="inlineStr">
-        <is>
-          <t>v3 6/2/24 TW</t>
-        </is>
-      </c>
-      <c r="C102" s="1521" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -33694,7 +33670,7 @@
     <mergeCell ref="K43:M43"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B1:I2"/>
-    <mergeCell ref="D98:E98"/>
+    <mergeCell ref="D97:E97"/>
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="C3:E4"/>
     <mergeCell ref="O72:R72"/>
@@ -33710,7 +33686,7 @@
     <mergeCell ref="K15:M15"/>
     <mergeCell ref="O62:R62"/>
     <mergeCell ref="F3:G4"/>
-    <mergeCell ref="D97:E97"/>
+    <mergeCell ref="D96:E96"/>
     <mergeCell ref="M9:O9"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="M1:R1"/>
@@ -33782,7 +33758,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M86">
+  <conditionalFormatting sqref="M85">
     <cfRule type="cellIs" rank="0" priority="17" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33793,12 +33769,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K86">
+  <conditionalFormatting sqref="K85">
     <cfRule type="cellIs" rank="0" priority="20" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M87">
+  <conditionalFormatting sqref="M86">
     <cfRule type="cellIs" rank="0" priority="21" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33809,12 +33785,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K87">
+  <conditionalFormatting sqref="K86">
     <cfRule type="cellIs" rank="0" priority="24" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M88:M89">
+  <conditionalFormatting sqref="M87:M88">
     <cfRule type="cellIs" rank="0" priority="25" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33825,29 +33801,13 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K88:K89">
+  <conditionalFormatting sqref="K87:K88">
     <cfRule type="cellIs" rank="0" priority="28" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M35">
     <cfRule type="cellIs" rank="0" priority="29" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="29" text="" percent="0" bottom="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M85">
-    <cfRule type="cellIs" rank="0" priority="30" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" rank="0" priority="31" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="31" text="" percent="0" bottom="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" rank="0" priority="32" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K85">
-    <cfRule type="cellIs" rank="0" priority="33" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -33861,7 +33821,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M50:M60 M62:M72 M83 M90:M95">
+  <conditionalFormatting sqref="M50:M60 M62:M72 M83 M89:M94">
     <cfRule type="cellIs" rank="0" priority="36" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33887,7 +33847,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K41 K44:K46 K90:K95 R61 R70:R71">
+  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K41 K44:K46 K89:K94 R61 R70:R71">
     <cfRule type="cellIs" rank="0" priority="42" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Afvulverslag: fust-volgorde afvul en verbruik gelijkgetrokken
Nieuwe volgorde (afvul rij 34-41, verbruik rij 85-92):
  20L KU Fust / 30L Jopen Fust / 50L Jopen Fust
  20L Gebr. Door Vrouwen Fust / 20L Other Fust / 20L KeyKeg / 30L KeyKeg

- Verbruik: elk fusttype eigen verliesregel tegen bijbehorende afvulrij
- Fustdop (rij 94): verlies t.o.v. de 5 stalen fusten (KeyKeg telde dubbel mee)
- KeyKegFustdop (rij 95): t.o.v. 20L + 30L KeyKeg
- Afvullen!C61: verlies alle 7 fusttypes
- 2 rijen ingevoegd; 'Ingevoerd in Mdrank' e.v. schuiven 2 rijen op
- formaten_field_map: 20L keykeg -> C40, 50L -> C36
- fix-american-dates.js: Afvulverslag!D97 -> D99

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CvHodB7rajqHXKYMVFnfMs
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -29784,7 +29784,7 @@
       </c>
       <c r="B61" s="2069" t="n"/>
       <c r="C61" s="2078">
-        <f>SUM(Afvulverslag!M85:M86)</f>
+        <f>SUM(Afvulverslag!M85:M87,Afvulverslag!M89:M92)</f>
         <v/>
       </c>
       <c r="D61" s="2070" t="n"/>
@@ -31093,7 +31093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R101"/>
+  <dimension ref="A1:R103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.00390625" defaultRowHeight="15" zeroHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="2.5" customWidth="1" style="2094" min="1" max="1"/>
@@ -32060,7 +32060,7 @@
     <row r="34" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B34" s="2013" t="inlineStr">
         <is>
-          <t>20L KeyKeg</t>
+          <t>20L KU Fust</t>
         </is>
       </c>
       <c r="C34" s="2149" t="n"/>
@@ -32084,7 +32084,7 @@
     <row r="35" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B35" s="2013" t="inlineStr">
         <is>
-          <t>20L KU Fust</t>
+          <t>30L Jopen Fust</t>
         </is>
       </c>
       <c r="C35" s="2149" t="n"/>
@@ -32101,23 +32101,23 @@
       </c>
       <c r="L35" s="2112" t="n"/>
       <c r="M35" s="2154">
-        <f>K35*20</f>
+        <f>K35*30</f>
         <v/>
       </c>
     </row>
     <row r="36" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B36" s="2013" t="inlineStr">
         <is>
-          <t>30L Jopen Fust</t>
-        </is>
-      </c>
-      <c r="C36" s="2158" t="n"/>
-      <c r="D36" s="2150" t="n"/>
-      <c r="E36" s="2151" t="n"/>
-      <c r="F36" s="2151" t="n"/>
-      <c r="G36" s="2151" t="n"/>
-      <c r="H36" s="2151" t="n"/>
-      <c r="I36" s="2150" t="n"/>
+          <t>50L Jopen Fust</t>
+        </is>
+      </c>
+      <c r="C36" s="2149" t="n"/>
+      <c r="D36" s="2160" t="n"/>
+      <c r="E36" s="2160" t="n"/>
+      <c r="F36" s="2160" t="n"/>
+      <c r="G36" s="2160" t="n"/>
+      <c r="H36" s="2160" t="n"/>
+      <c r="I36" s="2161" t="n"/>
       <c r="J36" s="1521" t="n"/>
       <c r="K36" s="2152">
         <f>SUM(D36:I36)</f>
@@ -32125,61 +32125,61 @@
       </c>
       <c r="L36" s="2112" t="n"/>
       <c r="M36" s="2154">
-        <f>K36*30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B37" s="2013" t="inlineStr">
-        <is>
-          <t>50L Jopen Fust</t>
-        </is>
-      </c>
-      <c r="C37" s="2149" t="n"/>
-      <c r="D37" s="2160" t="n"/>
-      <c r="E37" s="2160" t="n"/>
-      <c r="F37" s="2160" t="n"/>
-      <c r="G37" s="2160" t="n"/>
-      <c r="H37" s="2160" t="n"/>
-      <c r="I37" s="2161" t="n"/>
+        <f>K36*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B37" s="2162" t="n"/>
+      <c r="C37" s="1521" t="n"/>
+      <c r="D37" s="2163" t="n"/>
+      <c r="E37" s="2163" t="n"/>
+      <c r="F37" s="2163" t="n"/>
+      <c r="G37" s="2163" t="n"/>
+      <c r="H37" s="2163" t="n"/>
+      <c r="I37" s="2164" t="n"/>
       <c r="J37" s="1521" t="n"/>
-      <c r="K37" s="2152">
-        <f>SUM(D37:I37)</f>
-        <v/>
-      </c>
+      <c r="K37" s="2152" t="n"/>
       <c r="L37" s="2112" t="n"/>
-      <c r="M37" s="2154">
-        <f>K37*50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B38" s="2162" t="n"/>
+      <c r="M37" s="2154" t="n"/>
+    </row>
+    <row r="38" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B38" s="2013" t="inlineStr">
+        <is>
+          <t>20L Gebr. Door Vrouwen Fust</t>
+        </is>
+      </c>
       <c r="C38" s="1521" t="n"/>
-      <c r="D38" s="2163" t="n"/>
-      <c r="E38" s="2163" t="n"/>
-      <c r="F38" s="2163" t="n"/>
-      <c r="G38" s="2163" t="n"/>
-      <c r="H38" s="2163" t="n"/>
-      <c r="I38" s="2164" t="n"/>
+      <c r="D38" s="2165" t="n"/>
+      <c r="E38" s="2165" t="n"/>
+      <c r="F38" s="2165" t="n"/>
+      <c r="G38" s="2165" t="n"/>
+      <c r="H38" s="2165" t="n"/>
+      <c r="I38" s="2166" t="n"/>
       <c r="J38" s="1521" t="n"/>
-      <c r="K38" s="2152" t="n"/>
+      <c r="K38" s="2152">
+        <f>SUM(D38:I38)</f>
+        <v/>
+      </c>
       <c r="L38" s="2112" t="n"/>
-      <c r="M38" s="2154" t="n"/>
+      <c r="M38" s="2154">
+        <f>K38*20</f>
+        <v/>
+      </c>
     </row>
     <row r="39" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B39" s="2013" t="inlineStr">
         <is>
-          <t>20L Gbr. Door Vrouwen fust</t>
+          <t>20L Other Fust</t>
         </is>
       </c>
       <c r="C39" s="1521" t="n"/>
-      <c r="D39" s="2165" t="n"/>
-      <c r="E39" s="2165" t="n"/>
-      <c r="F39" s="2165" t="n"/>
-      <c r="G39" s="2165" t="n"/>
-      <c r="H39" s="2165" t="n"/>
-      <c r="I39" s="2166" t="n"/>
+      <c r="D39" s="2151" t="n"/>
+      <c r="E39" s="2151" t="n"/>
+      <c r="F39" s="2151" t="n"/>
+      <c r="G39" s="2151" t="n"/>
+      <c r="H39" s="2151" t="n"/>
+      <c r="I39" s="2150" t="n"/>
       <c r="J39" s="1521" t="n"/>
       <c r="K39" s="2152">
         <f>SUM(D39:I39)</f>
@@ -32194,7 +32194,7 @@
     <row r="40" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B40" s="2013" t="inlineStr">
         <is>
-          <t>20L Other kegs</t>
+          <t>20L KeyKeg</t>
         </is>
       </c>
       <c r="C40" s="1521" t="n"/>
@@ -33411,7 +33411,7 @@
     <row r="85" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B85" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 20L: </t>
+          <t>20L KU Fust</t>
         </is>
       </c>
       <c r="C85" s="1615" t="n"/>
@@ -33428,14 +33428,14 @@
       </c>
       <c r="L85" s="2112" t="n"/>
       <c r="M85" s="2152">
-        <f>K85-K35</f>
+        <f>K85-K34</f>
         <v/>
       </c>
     </row>
     <row r="86" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B86" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 30L: </t>
+          <t>30L Jopen Fust</t>
         </is>
       </c>
       <c r="C86" s="1615" t="n"/>
@@ -33445,21 +33445,21 @@
       <c r="G86" s="2184" t="n"/>
       <c r="H86" s="2184" t="n"/>
       <c r="I86" s="2184" t="n"/>
-      <c r="J86" s="2170" t="n"/>
+      <c r="J86" s="1521" t="n"/>
       <c r="K86" s="2152">
         <f>SUM(D86:I86)</f>
         <v/>
       </c>
       <c r="L86" s="2112" t="n"/>
       <c r="M86" s="2152">
-        <f>K86-K36</f>
+        <f>K86-K35</f>
         <v/>
       </c>
     </row>
     <row r="87" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B87" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jopen Fust 50L: </t>
+          <t>50L Jopen Fust</t>
         </is>
       </c>
       <c r="C87" s="1615" t="n"/>
@@ -33476,7 +33476,7 @@
       </c>
       <c r="L87" s="2112" t="n"/>
       <c r="M87" s="2152">
-        <f>K87-K37</f>
+        <f>K87-K36</f>
         <v/>
       </c>
     </row>
@@ -33497,7 +33497,7 @@
     <row r="89" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B89" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fustdop: </t>
+          <t>20L Gebr. Door Vrouwen Fust</t>
         </is>
       </c>
       <c r="C89" s="1615" t="n"/>
@@ -33514,37 +33514,47 @@
       </c>
       <c r="L89" s="2112" t="n"/>
       <c r="M89" s="2152">
-        <f>K89-SUM(K34:K37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B90" s="1099" t="n"/>
-      <c r="C90" s="2170" t="n"/>
-      <c r="D90" s="1521" t="n"/>
-      <c r="E90" s="1521" t="n"/>
-      <c r="F90" s="1521" t="n"/>
-      <c r="G90" s="1521" t="n"/>
-      <c r="H90" s="1521" t="n"/>
-      <c r="I90" s="1521" t="n"/>
-      <c r="J90" s="2170" t="n"/>
-      <c r="K90" s="2152" t="n"/>
+        <f>K89-K38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B90" s="2016" t="inlineStr">
+        <is>
+          <t>20L Other Fust</t>
+        </is>
+      </c>
+      <c r="C90" s="1615" t="n"/>
+      <c r="D90" s="2167" t="n"/>
+      <c r="E90" s="2184" t="n"/>
+      <c r="F90" s="2184" t="n"/>
+      <c r="G90" s="2184" t="n"/>
+      <c r="H90" s="2184" t="n"/>
+      <c r="I90" s="2184" t="n"/>
+      <c r="J90" s="1521" t="n"/>
+      <c r="K90" s="2152">
+        <f>SUM(D90:I90)</f>
+        <v/>
+      </c>
       <c r="L90" s="2112" t="n"/>
-      <c r="M90" s="2152" t="n"/>
+      <c r="M90" s="2152">
+        <f>K90-K39</f>
+        <v/>
+      </c>
     </row>
     <row r="91" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B91" s="2199" t="inlineStr">
-        <is>
-          <t>KeyKegFustdop:</t>
-        </is>
-      </c>
-      <c r="C91" s="2179" t="n"/>
-      <c r="D91" s="2193" t="n"/>
-      <c r="E91" s="2194" t="n"/>
-      <c r="F91" s="2194" t="n"/>
-      <c r="G91" s="2194" t="n"/>
-      <c r="H91" s="2194" t="n"/>
-      <c r="I91" s="2194" t="n"/>
+      <c r="B91" s="2016" t="inlineStr">
+        <is>
+          <t>20L KeyKeg</t>
+        </is>
+      </c>
+      <c r="C91" s="1615" t="n"/>
+      <c r="D91" s="2167" t="n"/>
+      <c r="E91" s="2184" t="n"/>
+      <c r="F91" s="2184" t="n"/>
+      <c r="G91" s="2184" t="n"/>
+      <c r="H91" s="2184" t="n"/>
+      <c r="I91" s="2184" t="n"/>
       <c r="J91" s="1521" t="n"/>
       <c r="K91" s="2152">
         <f>SUM(D91:I91)</f>
@@ -33552,23 +33562,23 @@
       </c>
       <c r="L91" s="2112" t="n"/>
       <c r="M91" s="2152">
-        <f>K91-K34-K41</f>
+        <f>K91-K40</f>
         <v/>
       </c>
     </row>
     <row r="92" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B92" s="2200" t="inlineStr">
-        <is>
-          <t>KeyKeg 20L - Leeg</t>
-        </is>
-      </c>
-      <c r="C92" s="2201" t="n"/>
-      <c r="D92" s="2202" t="n"/>
-      <c r="E92" s="2203" t="n"/>
-      <c r="F92" s="2203" t="n"/>
-      <c r="G92" s="2203" t="n"/>
-      <c r="H92" s="2203" t="n"/>
-      <c r="I92" s="2203" t="n"/>
+      <c r="B92" s="2016" t="inlineStr">
+        <is>
+          <t>30L KeyKeg</t>
+        </is>
+      </c>
+      <c r="C92" s="1615" t="n"/>
+      <c r="D92" s="2167" t="n"/>
+      <c r="E92" s="2184" t="n"/>
+      <c r="F92" s="2184" t="n"/>
+      <c r="G92" s="2184" t="n"/>
+      <c r="H92" s="2184" t="n"/>
+      <c r="I92" s="2184" t="n"/>
       <c r="J92" s="1521" t="n"/>
       <c r="K92" s="2152">
         <f>SUM(D92:I92)</f>
@@ -33576,80 +33586,102 @@
       </c>
       <c r="L92" s="2112" t="n"/>
       <c r="M92" s="2152">
-        <f>K92-K34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B93" s="2016" t="inlineStr">
-        <is>
-          <t>KeyKeg 30L - Leeg</t>
-        </is>
-      </c>
-      <c r="C93" s="2204" t="n"/>
-      <c r="D93" s="2160" t="n"/>
-      <c r="E93" s="2161" t="n"/>
-      <c r="F93" s="2161" t="n"/>
-      <c r="G93" s="2161" t="n"/>
-      <c r="H93" s="2161" t="n"/>
-      <c r="I93" s="2161" t="n"/>
+        <f>K92-K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B93" s="2185" t="n"/>
+      <c r="C93" s="2198" t="n"/>
+      <c r="D93" s="2156" t="n"/>
+      <c r="E93" s="2156" t="n"/>
+      <c r="F93" s="2156" t="n"/>
+      <c r="G93" s="2156" t="n"/>
+      <c r="H93" s="2156" t="n"/>
+      <c r="I93" s="2156" t="n"/>
       <c r="J93" s="1521" t="n"/>
-      <c r="K93" s="2152">
-        <f>SUM(D93:I93)</f>
-        <v/>
-      </c>
+      <c r="K93" s="2152" t="n"/>
       <c r="L93" s="2112" t="n"/>
-      <c r="M93" s="2152">
-        <f>K93-K41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" ht="15" customHeight="1" s="1339"/>
-    <row r="95" ht="15" customHeight="1" s="1339"/>
-    <row r="96" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B96" s="2013" t="inlineStr">
+      <c r="M93" s="2152" t="n"/>
+    </row>
+    <row r="94" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B94" s="2016" t="inlineStr">
+        <is>
+          <t>Fustdop:</t>
+        </is>
+      </c>
+      <c r="C94" s="1615" t="n"/>
+      <c r="D94" s="2167" t="n"/>
+      <c r="E94" s="2184" t="n"/>
+      <c r="F94" s="2184" t="n"/>
+      <c r="G94" s="2184" t="n"/>
+      <c r="H94" s="2184" t="n"/>
+      <c r="I94" s="2184" t="n"/>
+      <c r="J94" s="1521" t="n"/>
+      <c r="K94" s="2152">
+        <f>SUM(D94:I94)</f>
+        <v/>
+      </c>
+      <c r="L94" s="2112" t="n"/>
+      <c r="M94" s="2152">
+        <f>K94-K34-K35-K36-K38-K39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B95" s="2016" t="inlineStr">
+        <is>
+          <t>KeyKegFustdop:</t>
+        </is>
+      </c>
+      <c r="C95" s="2204" t="n"/>
+      <c r="D95" s="2160" t="n"/>
+      <c r="E95" s="2161" t="n"/>
+      <c r="F95" s="2161" t="n"/>
+      <c r="G95" s="2161" t="n"/>
+      <c r="H95" s="2161" t="n"/>
+      <c r="I95" s="2161" t="n"/>
+      <c r="J95" s="1521" t="n"/>
+      <c r="K95" s="2152">
+        <f>SUM(D95:I95)</f>
+        <v/>
+      </c>
+      <c r="L95" s="2112" t="n"/>
+      <c r="M95" s="2152">
+        <f>K95-K40-K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" ht="15" customHeight="1" s="1339"/>
+    <row r="97" ht="15" customHeight="1" s="1339"/>
+    <row r="98" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B98" s="2013" t="inlineStr">
         <is>
           <t>Ingevoerd in Mdrank</t>
         </is>
       </c>
-      <c r="C96" s="2026" t="inlineStr">
+      <c r="C98" s="2026" t="inlineStr">
         <is>
           <t>door:</t>
         </is>
       </c>
-      <c r="D96" s="2205" t="n"/>
-      <c r="E96" s="1115" t="n"/>
-    </row>
-    <row r="97" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B97" s="2206" t="n"/>
-      <c r="C97" s="2026" t="inlineStr">
+      <c r="D98" s="2205" t="n"/>
+      <c r="E98" s="1115" t="n"/>
+    </row>
+    <row r="99" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B99" s="2206" t="n"/>
+      <c r="C99" s="2026" t="inlineStr">
         <is>
           <t>datum:</t>
         </is>
       </c>
-      <c r="D97" s="2215" t="n"/>
-      <c r="E97" s="1115" t="n"/>
-    </row>
-    <row r="98" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B98" s="2208" t="inlineStr">
-        <is>
-          <t>V2,1 : 09-10-17 KYT</t>
-        </is>
-      </c>
-      <c r="C98" s="1521" t="n"/>
-    </row>
-    <row r="99" ht="15" customFormat="1" customHeight="1" s="1425">
-      <c r="B99" s="2208" t="inlineStr">
-        <is>
-          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
-        </is>
-      </c>
-      <c r="C99" s="1521" t="n"/>
+      <c r="D99" s="2215" t="n"/>
+      <c r="E99" s="1115" t="n"/>
     </row>
     <row r="100" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B100" s="2208" t="inlineStr">
         <is>
-          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
+          <t>V2,1 : 09-10-17 KYT</t>
         </is>
       </c>
       <c r="C100" s="1521" t="n"/>
@@ -33657,10 +33689,26 @@
     <row r="101" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B101" s="2208" t="inlineStr">
         <is>
+          <t>V2,001 : 02/10/2017 KYT, invoeg MR-Opdracht</t>
+        </is>
+      </c>
+      <c r="C101" s="1521" t="n"/>
+    </row>
+    <row r="102" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B102" s="2208" t="inlineStr">
+        <is>
+          <t>V2,002 : 22/11/2018 KYT: nav MvdG&amp;JL</t>
+        </is>
+      </c>
+      <c r="C102" s="1521" t="n"/>
+    </row>
+    <row r="103" ht="15" customFormat="1" customHeight="1" s="1425">
+      <c r="B103" s="2208" t="inlineStr">
+        <is>
           <t>v3 6/2/24 TW</t>
         </is>
       </c>
-      <c r="C101" s="1521" t="n"/>
+      <c r="C103" s="1521" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -33670,7 +33718,7 @@
     <mergeCell ref="K43:M43"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B1:I2"/>
-    <mergeCell ref="D97:E97"/>
+    <mergeCell ref="D99:E99"/>
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="C3:E4"/>
     <mergeCell ref="O72:R72"/>
@@ -33686,7 +33734,7 @@
     <mergeCell ref="K15:M15"/>
     <mergeCell ref="O62:R62"/>
     <mergeCell ref="F3:G4"/>
-    <mergeCell ref="D96:E96"/>
+    <mergeCell ref="D98:E98"/>
     <mergeCell ref="M9:O9"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="M1:R1"/>
@@ -33821,7 +33869,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M50:M60 M62:M72 M83 M89:M94">
+  <conditionalFormatting sqref="M50:M60 M62:M72 M83 M89:M96">
     <cfRule type="cellIs" rank="0" priority="36" equalAverage="0" operator="equal" aboveAverage="0" dxfId="30" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>
@@ -33847,7 +33895,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K41 K44:K46 K89:K94 R61 R70:R71">
+  <conditionalFormatting sqref="K17:K18 K20:K21 K23:K25 K34:K41 K44:K46 K89:K96 R61 R70:R71">
     <cfRule type="cellIs" rank="0" priority="42" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Filling Report: omdozen weer 'Blanco' i.p.v. 'Blank'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CvHodB7rajqHXKYMVFnfMs
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -32604,7 +32604,7 @@
     <row r="56" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B56" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 24x33cl - Blank</t>
+          <t xml:space="preserve">Outer Box 24x33cl - Blanco</t>
         </is>
       </c>
       <c r="C56" s="2180" t="n"/>
@@ -32678,7 +32678,7 @@
     <row r="59" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B59" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 12x33cl - Blank</t>
+          <t xml:space="preserve">Outer Box 12x33cl - Blanco</t>
         </is>
       </c>
       <c r="C59" s="2180" t="n"/>
@@ -32912,7 +32912,7 @@
     <row r="68" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B68" s="2016" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 6x75cl - Blank</t>
+          <t xml:space="preserve">Outer Box 6x75cl - Blanco</t>
         </is>
       </c>
       <c r="C68" s="2188" t="n"/>
@@ -33251,7 +33251,7 @@
     <row r="79" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B79" s="2192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 12x33cl Can - Blank</t>
+          <t xml:space="preserve">Outer Box 12x33cl Can - Blanco</t>
         </is>
       </c>
       <c r="C79" s="1615" t="n"/>
@@ -33280,7 +33280,7 @@
     <row r="80" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B80" s="2192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 24x33cl Can - Blank</t>
+          <t xml:space="preserve">Outer Box 24x33cl Can - Blanco</t>
         </is>
       </c>
       <c r="C80" s="1615" t="n"/>
@@ -33301,7 +33301,7 @@
     <row r="81" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B81" s="2192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 12x44cl Can - Blank</t>
+          <t xml:space="preserve">Outer Box 12x44cl Can - Blanco</t>
         </is>
       </c>
       <c r="C81" s="1615" t="n"/>
@@ -33322,7 +33322,7 @@
     <row r="82" outlineLevel="1" ht="15" customFormat="1" customHeight="1" s="1425">
       <c r="B82" s="2192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outer Box 24x44cl Can - Blank</t>
+          <t xml:space="preserve">Outer Box 24x44cl Can - Blanco</t>
         </is>
       </c>
       <c r="C82" s="1615" t="n"/>

</xml_diff>